<commit_message>
Auto-derive context-questions-per-thread (C) via session gap analysis
ユーザーから update_shukei.py の仕様を教えてもらい、業務削減効果_試算の
「1つの文脈での質問数(C)」を再現できるようになった。ユーザーごとに
発言間隔が60分を超えたら新セッションとみなしてセッション数を数え、
総プロンプト数÷セッション数でCを算出する。実データ検証で C=4.104
(参照ファイルの4.109とほぼ一致)。これで全シートが生ログから完全自動で
再構築可能になった。

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01598FP6oS2STFUTDPWRj1o6
</commit_message>
<xml_diff>
--- a/QommonsAI利用集計.xlsx
+++ b/QommonsAI利用集計.xlsx
@@ -59809,7 +59809,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>4.109</v>
+        <v>4.104</v>
       </c>
       <c r="C29">
         <f>ROUND(C28/B29,0)</f>
@@ -59866,7 +59866,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>【前提】入出力文字数はログ集計値（プレフィックス除く）。質問数Cは会話スレッドIDが生ログに無いため自動再計算していません。実測し直す場合はこの値を編集してください。</t>
+          <t>【前提】入出力文字数はログ集計値（プレフィックス除く）。質問数C=総プロンプト数÷セッション数(ユーザーごとに発言間隔が60分を超えたら新セッション、として自動算出。今回のセッション数=3834)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Base department usage_rate on 利用開始済み(status=完了) registrants
「未完了」はアカウント発行済みだが未利用の登録者(ユーザー確認済み)。
これを利用率の分母に含めると、まだ使い始めていない人のせいで実際の
定着率が過小評価されるため、分母を「完了」ステータスの登録者数に変更。
部署別集計シートに 登録者数(全体) と 登録者数(利用開始済み) を併記する。

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01598FP6oS2STFUTDPWRj1o6
</commit_message>
<xml_diff>
--- a/QommonsAI利用集計.xlsx
+++ b/QommonsAI利用集計.xlsx
@@ -457,18 +457,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I140"/>
+  <dimension ref="A1:J140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="9" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -481,7 +482,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>集計期間: 2026-07-01 〜 2026-07-21  ／ 利用回数=プロンプト(質問)数  ／ 使用文字数=入力+出力(プレフィックス除く)</t>
+          <t>集計期間: 2026-07-01 〜 2026-07-21  ／ 利用回数=プロンプト(質問)数  ／ 使用文字数=入力+出力(プレフィックス除く)  ／ 利用率=利用者数÷登録者数(利用開始済み)</t>
         </is>
       </c>
     </row>
@@ -493,40 +494,47 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>登録者数</t>
+          <t>登録者数
+(全体)</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
+          <t>登録者数
+(利用開始済み)</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
           <t>利用者数</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>利用率</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>プロンプト数</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>応答数</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>合計レコード</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>使用文字数</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>1人あたり
 プロンプト数(利用者)</t>
@@ -543,24 +551,27 @@
         <v>10</v>
       </c>
       <c r="C5" t="n">
+        <v>10</v>
+      </c>
+      <c r="D5" t="n">
         <v>11</v>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="E5" s="4" t="n">
         <v>1.1</v>
       </c>
-      <c r="E5" t="n">
+      <c r="F5" t="n">
         <v>1001</v>
       </c>
-      <c r="F5" t="n">
+      <c r="G5" t="n">
         <v>980</v>
       </c>
-      <c r="G5" t="n">
+      <c r="H5" t="n">
         <v>1981</v>
       </c>
-      <c r="H5" t="n">
+      <c r="I5" t="n">
         <v>1779787</v>
       </c>
-      <c r="I5" t="n">
+      <c r="J5" t="n">
         <v>91</v>
       </c>
     </row>
@@ -576,22 +587,25 @@
       <c r="C6" t="n">
         <v>11</v>
       </c>
-      <c r="D6" s="4" t="n">
-        <v>0.8461538461538461</v>
-      </c>
-      <c r="E6" t="n">
+      <c r="D6" t="n">
+        <v>11</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" t="n">
         <v>982</v>
       </c>
-      <c r="F6" t="n">
+      <c r="G6" t="n">
         <v>971</v>
       </c>
-      <c r="G6" t="n">
+      <c r="H6" t="n">
         <v>1953</v>
       </c>
-      <c r="H6" t="n">
+      <c r="I6" t="n">
         <v>1170131</v>
       </c>
-      <c r="I6" t="n">
+      <c r="J6" t="n">
         <v>89</v>
       </c>
     </row>
@@ -605,24 +619,27 @@
         <v>8</v>
       </c>
       <c r="C7" t="n">
+        <v>8</v>
+      </c>
+      <c r="D7" t="n">
         <v>6</v>
       </c>
-      <c r="D7" s="4" t="n">
+      <c r="E7" s="4" t="n">
         <v>0.75</v>
       </c>
-      <c r="E7" t="n">
+      <c r="F7" t="n">
         <v>782</v>
       </c>
-      <c r="F7" t="n">
+      <c r="G7" t="n">
         <v>771</v>
       </c>
-      <c r="G7" t="n">
+      <c r="H7" t="n">
         <v>1553</v>
       </c>
-      <c r="H7" t="n">
+      <c r="I7" t="n">
         <v>1234438</v>
       </c>
-      <c r="I7" t="n">
+      <c r="J7" t="n">
         <v>130</v>
       </c>
     </row>
@@ -638,22 +655,25 @@
       <c r="C8" t="n">
         <v>10</v>
       </c>
-      <c r="D8" s="4" t="n">
-        <v>0.8333333333333334</v>
-      </c>
-      <c r="E8" t="n">
+      <c r="D8" t="n">
+        <v>10</v>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" t="n">
         <v>699</v>
       </c>
-      <c r="F8" t="n">
+      <c r="G8" t="n">
         <v>693</v>
       </c>
-      <c r="G8" t="n">
+      <c r="H8" t="n">
         <v>1392</v>
       </c>
-      <c r="H8" t="n">
+      <c r="I8" t="n">
         <v>1054378</v>
       </c>
-      <c r="I8" t="n">
+      <c r="J8" t="n">
         <v>70</v>
       </c>
     </row>
@@ -667,24 +687,27 @@
         <v>17</v>
       </c>
       <c r="C9" t="n">
+        <v>16</v>
+      </c>
+      <c r="D9" t="n">
         <v>12</v>
       </c>
-      <c r="D9" s="4" t="n">
-        <v>0.7058823529411765</v>
-      </c>
-      <c r="E9" t="n">
+      <c r="E9" s="4" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="F9" t="n">
         <v>583</v>
       </c>
-      <c r="F9" t="n">
+      <c r="G9" t="n">
         <v>580</v>
       </c>
-      <c r="G9" t="n">
+      <c r="H9" t="n">
         <v>1163</v>
       </c>
-      <c r="H9" t="n">
+      <c r="I9" t="n">
         <v>898619</v>
       </c>
-      <c r="I9" t="n">
+      <c r="J9" t="n">
         <v>49</v>
       </c>
     </row>
@@ -698,24 +721,27 @@
         <v>30</v>
       </c>
       <c r="C10" t="n">
+        <v>21</v>
+      </c>
+      <c r="D10" t="n">
         <v>17</v>
       </c>
-      <c r="D10" s="4" t="n">
-        <v>0.5666666666666667</v>
-      </c>
-      <c r="E10" t="n">
+      <c r="E10" s="4" t="n">
+        <v>0.8095238095238095</v>
+      </c>
+      <c r="F10" t="n">
         <v>536</v>
       </c>
-      <c r="F10" t="n">
+      <c r="G10" t="n">
         <v>532</v>
       </c>
-      <c r="G10" t="n">
+      <c r="H10" t="n">
         <v>1068</v>
       </c>
-      <c r="H10" t="n">
+      <c r="I10" t="n">
         <v>842215</v>
       </c>
-      <c r="I10" t="n">
+      <c r="J10" t="n">
         <v>32</v>
       </c>
     </row>
@@ -731,22 +757,25 @@
       <c r="C11" t="n">
         <v>7</v>
       </c>
-      <c r="D11" s="4" t="n">
+      <c r="D11" t="n">
+        <v>7</v>
+      </c>
+      <c r="E11" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="E11" t="n">
+      <c r="F11" t="n">
         <v>492</v>
       </c>
-      <c r="F11" t="n">
+      <c r="G11" t="n">
         <v>487</v>
       </c>
-      <c r="G11" t="n">
+      <c r="H11" t="n">
         <v>979</v>
       </c>
-      <c r="H11" t="n">
+      <c r="I11" t="n">
         <v>748956</v>
       </c>
-      <c r="I11" t="n">
+      <c r="J11" t="n">
         <v>70</v>
       </c>
     </row>
@@ -762,22 +791,25 @@
       <c r="C12" t="n">
         <v>5</v>
       </c>
-      <c r="D12" s="4" t="n">
-        <v>0.5555555555555556</v>
-      </c>
-      <c r="E12" t="n">
+      <c r="D12" t="n">
+        <v>5</v>
+      </c>
+      <c r="E12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" t="n">
         <v>433</v>
       </c>
-      <c r="F12" t="n">
+      <c r="G12" t="n">
         <v>430</v>
       </c>
-      <c r="G12" t="n">
+      <c r="H12" t="n">
         <v>863</v>
       </c>
-      <c r="H12" t="n">
+      <c r="I12" t="n">
         <v>760047</v>
       </c>
-      <c r="I12" t="n">
+      <c r="J12" t="n">
         <v>87</v>
       </c>
     </row>
@@ -791,24 +823,27 @@
         <v>16</v>
       </c>
       <c r="C13" t="n">
+        <v>15</v>
+      </c>
+      <c r="D13" t="n">
         <v>13</v>
       </c>
-      <c r="D13" s="4" t="n">
-        <v>0.8125</v>
-      </c>
-      <c r="E13" t="n">
+      <c r="E13" s="4" t="n">
+        <v>0.8666666666666667</v>
+      </c>
+      <c r="F13" t="n">
         <v>426</v>
       </c>
-      <c r="F13" t="n">
+      <c r="G13" t="n">
         <v>425</v>
       </c>
-      <c r="G13" t="n">
+      <c r="H13" t="n">
         <v>851</v>
       </c>
-      <c r="H13" t="n">
+      <c r="I13" t="n">
         <v>657292</v>
       </c>
-      <c r="I13" t="n">
+      <c r="J13" t="n">
         <v>33</v>
       </c>
     </row>
@@ -824,22 +859,25 @@
       <c r="C14" t="n">
         <v>3</v>
       </c>
-      <c r="D14" s="4" t="n">
-        <v>0.4285714285714285</v>
-      </c>
-      <c r="E14" t="n">
+      <c r="D14" t="n">
+        <v>3</v>
+      </c>
+      <c r="E14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" t="n">
         <v>416</v>
       </c>
-      <c r="F14" t="n">
+      <c r="G14" t="n">
         <v>407</v>
       </c>
-      <c r="G14" t="n">
+      <c r="H14" t="n">
         <v>823</v>
       </c>
-      <c r="H14" t="n">
+      <c r="I14" t="n">
         <v>563572</v>
       </c>
-      <c r="I14" t="n">
+      <c r="J14" t="n">
         <v>139</v>
       </c>
     </row>
@@ -855,22 +893,25 @@
       <c r="C15" t="n">
         <v>6</v>
       </c>
-      <c r="D15" s="4" t="n">
-        <v>0.8571428571428571</v>
-      </c>
-      <c r="E15" t="n">
+      <c r="D15" t="n">
+        <v>6</v>
+      </c>
+      <c r="E15" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" t="n">
         <v>371</v>
       </c>
-      <c r="F15" t="n">
+      <c r="G15" t="n">
         <v>368</v>
       </c>
-      <c r="G15" t="n">
+      <c r="H15" t="n">
         <v>739</v>
       </c>
-      <c r="H15" t="n">
+      <c r="I15" t="n">
         <v>481829</v>
       </c>
-      <c r="I15" t="n">
+      <c r="J15" t="n">
         <v>62</v>
       </c>
     </row>
@@ -884,24 +925,27 @@
         <v>12</v>
       </c>
       <c r="C16" t="n">
+        <v>9</v>
+      </c>
+      <c r="D16" t="n">
         <v>8</v>
       </c>
-      <c r="D16" s="4" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="E16" t="n">
+      <c r="E16" s="4" t="n">
+        <v>0.8888888888888888</v>
+      </c>
+      <c r="F16" t="n">
         <v>343</v>
       </c>
-      <c r="F16" t="n">
+      <c r="G16" t="n">
         <v>336</v>
       </c>
-      <c r="G16" t="n">
+      <c r="H16" t="n">
         <v>679</v>
       </c>
-      <c r="H16" t="n">
+      <c r="I16" t="n">
         <v>516173</v>
       </c>
-      <c r="I16" t="n">
+      <c r="J16" t="n">
         <v>43</v>
       </c>
     </row>
@@ -917,22 +961,25 @@
       <c r="C17" t="n">
         <v>8</v>
       </c>
-      <c r="D17" s="4" t="n">
-        <v>0.8888888888888888</v>
-      </c>
-      <c r="E17" t="n">
+      <c r="D17" t="n">
+        <v>8</v>
+      </c>
+      <c r="E17" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" t="n">
         <v>331</v>
       </c>
-      <c r="F17" t="n">
+      <c r="G17" t="n">
         <v>330</v>
       </c>
-      <c r="G17" t="n">
+      <c r="H17" t="n">
         <v>661</v>
       </c>
-      <c r="H17" t="n">
+      <c r="I17" t="n">
         <v>525196</v>
       </c>
-      <c r="I17" t="n">
+      <c r="J17" t="n">
         <v>41</v>
       </c>
     </row>
@@ -948,22 +995,25 @@
       <c r="C18" t="n">
         <v>1</v>
       </c>
-      <c r="D18" s="4" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E18" t="n">
+      <c r="D18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" t="n">
         <v>314</v>
       </c>
-      <c r="F18" t="n">
+      <c r="G18" t="n">
         <v>312</v>
       </c>
-      <c r="G18" t="n">
+      <c r="H18" t="n">
         <v>626</v>
       </c>
-      <c r="H18" t="n">
+      <c r="I18" t="n">
         <v>404145</v>
       </c>
-      <c r="I18" t="n">
+      <c r="J18" t="n">
         <v>314</v>
       </c>
     </row>
@@ -977,24 +1027,27 @@
         <v>13</v>
       </c>
       <c r="C19" t="n">
+        <v>11</v>
+      </c>
+      <c r="D19" t="n">
         <v>9</v>
       </c>
-      <c r="D19" s="4" t="n">
-        <v>0.6923076923076923</v>
-      </c>
-      <c r="E19" t="n">
+      <c r="E19" s="4" t="n">
+        <v>0.8181818181818182</v>
+      </c>
+      <c r="F19" t="n">
         <v>308</v>
       </c>
-      <c r="F19" t="n">
+      <c r="G19" t="n">
         <v>305</v>
       </c>
-      <c r="G19" t="n">
+      <c r="H19" t="n">
         <v>613</v>
       </c>
-      <c r="H19" t="n">
+      <c r="I19" t="n">
         <v>295382</v>
       </c>
-      <c r="I19" t="n">
+      <c r="J19" t="n">
         <v>34</v>
       </c>
     </row>
@@ -1010,22 +1063,25 @@
       <c r="C20" t="n">
         <v>7</v>
       </c>
-      <c r="D20" s="4" t="n">
+      <c r="D20" t="n">
+        <v>7</v>
+      </c>
+      <c r="E20" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="E20" t="n">
+      <c r="F20" t="n">
         <v>303</v>
       </c>
-      <c r="F20" t="n">
+      <c r="G20" t="n">
         <v>299</v>
       </c>
-      <c r="G20" t="n">
+      <c r="H20" t="n">
         <v>602</v>
       </c>
-      <c r="H20" t="n">
+      <c r="I20" t="n">
         <v>449750</v>
       </c>
-      <c r="I20" t="n">
+      <c r="J20" t="n">
         <v>43</v>
       </c>
     </row>
@@ -1039,24 +1095,27 @@
         <v>11</v>
       </c>
       <c r="C21" t="n">
+        <v>10</v>
+      </c>
+      <c r="D21" t="n">
         <v>8</v>
       </c>
-      <c r="D21" s="4" t="n">
-        <v>0.7272727272727273</v>
-      </c>
-      <c r="E21" t="n">
+      <c r="E21" s="4" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F21" t="n">
         <v>288</v>
       </c>
-      <c r="F21" t="n">
+      <c r="G21" t="n">
         <v>285</v>
       </c>
-      <c r="G21" t="n">
+      <c r="H21" t="n">
         <v>573</v>
       </c>
-      <c r="H21" t="n">
+      <c r="I21" t="n">
         <v>417501</v>
       </c>
-      <c r="I21" t="n">
+      <c r="J21" t="n">
         <v>36</v>
       </c>
     </row>
@@ -1070,24 +1129,27 @@
         <v>25</v>
       </c>
       <c r="C22" t="n">
+        <v>16</v>
+      </c>
+      <c r="D22" t="n">
         <v>9</v>
       </c>
-      <c r="D22" s="4" t="n">
-        <v>0.36</v>
-      </c>
-      <c r="E22" t="n">
+      <c r="E22" s="4" t="n">
+        <v>0.5625</v>
+      </c>
+      <c r="F22" t="n">
         <v>253</v>
       </c>
-      <c r="F22" t="n">
+      <c r="G22" t="n">
         <v>251</v>
       </c>
-      <c r="G22" t="n">
+      <c r="H22" t="n">
         <v>504</v>
       </c>
-      <c r="H22" t="n">
+      <c r="I22" t="n">
         <v>347196</v>
       </c>
-      <c r="I22" t="n">
+      <c r="J22" t="n">
         <v>28</v>
       </c>
     </row>
@@ -1101,24 +1163,27 @@
         <v>7</v>
       </c>
       <c r="C23" t="n">
+        <v>5</v>
+      </c>
+      <c r="D23" t="n">
         <v>4</v>
       </c>
-      <c r="D23" s="4" t="n">
-        <v>0.5714285714285714</v>
-      </c>
-      <c r="E23" t="n">
+      <c r="E23" s="4" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F23" t="n">
         <v>245</v>
       </c>
-      <c r="F23" t="n">
+      <c r="G23" t="n">
         <v>242</v>
       </c>
-      <c r="G23" t="n">
+      <c r="H23" t="n">
         <v>487</v>
       </c>
-      <c r="H23" t="n">
+      <c r="I23" t="n">
         <v>334187</v>
       </c>
-      <c r="I23" t="n">
+      <c r="J23" t="n">
         <v>61</v>
       </c>
     </row>
@@ -1132,24 +1197,27 @@
         <v>8</v>
       </c>
       <c r="C24" t="n">
+        <v>6</v>
+      </c>
+      <c r="D24" t="n">
         <v>5</v>
       </c>
-      <c r="D24" s="4" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="E24" t="n">
+      <c r="E24" s="4" t="n">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="F24" t="n">
         <v>232</v>
       </c>
-      <c r="F24" t="n">
+      <c r="G24" t="n">
         <v>231</v>
       </c>
-      <c r="G24" t="n">
+      <c r="H24" t="n">
         <v>463</v>
       </c>
-      <c r="H24" t="n">
+      <c r="I24" t="n">
         <v>370708</v>
       </c>
-      <c r="I24" t="n">
+      <c r="J24" t="n">
         <v>46</v>
       </c>
     </row>
@@ -1165,22 +1233,25 @@
       <c r="C25" t="n">
         <v>4</v>
       </c>
-      <c r="D25" s="4" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="E25" t="n">
+      <c r="D25" t="n">
+        <v>4</v>
+      </c>
+      <c r="E25" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" t="n">
         <v>229</v>
       </c>
-      <c r="F25" t="n">
+      <c r="G25" t="n">
         <v>225</v>
       </c>
-      <c r="G25" t="n">
+      <c r="H25" t="n">
         <v>454</v>
       </c>
-      <c r="H25" t="n">
+      <c r="I25" t="n">
         <v>307643</v>
       </c>
-      <c r="I25" t="n">
+      <c r="J25" t="n">
         <v>57</v>
       </c>
     </row>
@@ -1194,24 +1265,27 @@
         <v>21</v>
       </c>
       <c r="C26" t="n">
+        <v>16</v>
+      </c>
+      <c r="D26" t="n">
         <v>12</v>
       </c>
-      <c r="D26" s="4" t="n">
-        <v>0.5714285714285714</v>
-      </c>
-      <c r="E26" t="n">
+      <c r="E26" s="4" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="F26" t="n">
         <v>224</v>
       </c>
-      <c r="F26" t="n">
+      <c r="G26" t="n">
         <v>221</v>
       </c>
-      <c r="G26" t="n">
+      <c r="H26" t="n">
         <v>445</v>
       </c>
-      <c r="H26" t="n">
+      <c r="I26" t="n">
         <v>307184</v>
       </c>
-      <c r="I26" t="n">
+      <c r="J26" t="n">
         <v>19</v>
       </c>
     </row>
@@ -1225,24 +1299,27 @@
         <v>18</v>
       </c>
       <c r="C27" t="n">
+        <v>11</v>
+      </c>
+      <c r="D27" t="n">
         <v>9</v>
       </c>
-      <c r="D27" s="4" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E27" t="n">
+      <c r="E27" s="4" t="n">
+        <v>0.8181818181818182</v>
+      </c>
+      <c r="F27" t="n">
         <v>212</v>
       </c>
-      <c r="F27" t="n">
+      <c r="G27" t="n">
         <v>210</v>
       </c>
-      <c r="G27" t="n">
+      <c r="H27" t="n">
         <v>422</v>
       </c>
-      <c r="H27" t="n">
+      <c r="I27" t="n">
         <v>236511</v>
       </c>
-      <c r="I27" t="n">
+      <c r="J27" t="n">
         <v>24</v>
       </c>
     </row>
@@ -1256,24 +1333,27 @@
         <v>10</v>
       </c>
       <c r="C28" t="n">
+        <v>8</v>
+      </c>
+      <c r="D28" t="n">
         <v>5</v>
       </c>
-      <c r="D28" s="4" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E28" t="n">
+      <c r="E28" s="4" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="F28" t="n">
         <v>192</v>
       </c>
-      <c r="F28" t="n">
+      <c r="G28" t="n">
         <v>189</v>
       </c>
-      <c r="G28" t="n">
+      <c r="H28" t="n">
         <v>381</v>
       </c>
-      <c r="H28" t="n">
+      <c r="I28" t="n">
         <v>280997</v>
       </c>
-      <c r="I28" t="n">
+      <c r="J28" t="n">
         <v>38</v>
       </c>
     </row>
@@ -1287,24 +1367,27 @@
         <v>6</v>
       </c>
       <c r="C29" t="n">
+        <v>6</v>
+      </c>
+      <c r="D29" t="n">
         <v>5</v>
       </c>
-      <c r="D29" s="4" t="n">
+      <c r="E29" s="4" t="n">
         <v>0.8333333333333334</v>
       </c>
-      <c r="E29" t="n">
+      <c r="F29" t="n">
         <v>185</v>
       </c>
-      <c r="F29" t="n">
+      <c r="G29" t="n">
         <v>181</v>
       </c>
-      <c r="G29" t="n">
+      <c r="H29" t="n">
         <v>366</v>
       </c>
-      <c r="H29" t="n">
+      <c r="I29" t="n">
         <v>341325</v>
       </c>
-      <c r="I29" t="n">
+      <c r="J29" t="n">
         <v>37</v>
       </c>
     </row>
@@ -1318,24 +1401,27 @@
         <v>7</v>
       </c>
       <c r="C30" t="n">
+        <v>6</v>
+      </c>
+      <c r="D30" t="n">
         <v>5</v>
       </c>
-      <c r="D30" s="4" t="n">
-        <v>0.7142857142857143</v>
-      </c>
-      <c r="E30" t="n">
+      <c r="E30" s="4" t="n">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="F30" t="n">
         <v>154</v>
       </c>
-      <c r="F30" t="n">
+      <c r="G30" t="n">
         <v>151</v>
       </c>
-      <c r="G30" t="n">
+      <c r="H30" t="n">
         <v>305</v>
       </c>
-      <c r="H30" t="n">
+      <c r="I30" t="n">
         <v>254351</v>
       </c>
-      <c r="I30" t="n">
+      <c r="J30" t="n">
         <v>31</v>
       </c>
     </row>
@@ -1351,22 +1437,25 @@
       <c r="C31" t="n">
         <v>2</v>
       </c>
-      <c r="D31" s="4" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="E31" t="n">
+      <c r="D31" t="n">
+        <v>2</v>
+      </c>
+      <c r="E31" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F31" t="n">
         <v>145</v>
       </c>
-      <c r="F31" t="n">
+      <c r="G31" t="n">
         <v>142</v>
       </c>
-      <c r="G31" t="n">
+      <c r="H31" t="n">
         <v>287</v>
       </c>
-      <c r="H31" t="n">
+      <c r="I31" t="n">
         <v>249255</v>
       </c>
-      <c r="I31" t="n">
+      <c r="J31" t="n">
         <v>72</v>
       </c>
     </row>
@@ -1382,22 +1471,25 @@
       <c r="C32" t="n">
         <v>6</v>
       </c>
-      <c r="D32" s="4" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="E32" t="n">
+      <c r="D32" t="n">
+        <v>6</v>
+      </c>
+      <c r="E32" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F32" t="n">
         <v>134</v>
       </c>
-      <c r="F32" t="n">
+      <c r="G32" t="n">
         <v>133</v>
       </c>
-      <c r="G32" t="n">
+      <c r="H32" t="n">
         <v>267</v>
       </c>
-      <c r="H32" t="n">
+      <c r="I32" t="n">
         <v>179880</v>
       </c>
-      <c r="I32" t="n">
+      <c r="J32" t="n">
         <v>22</v>
       </c>
     </row>
@@ -1411,24 +1503,27 @@
         <v>4</v>
       </c>
       <c r="C33" t="n">
+        <v>2</v>
+      </c>
+      <c r="D33" t="n">
         <v>1</v>
       </c>
-      <c r="D33" s="4" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="E33" t="n">
+      <c r="E33" s="4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F33" t="n">
         <v>130</v>
       </c>
-      <c r="F33" t="n">
+      <c r="G33" t="n">
         <v>127</v>
       </c>
-      <c r="G33" t="n">
+      <c r="H33" t="n">
         <v>257</v>
       </c>
-      <c r="H33" t="n">
+      <c r="I33" t="n">
         <v>236039</v>
       </c>
-      <c r="I33" t="n">
+      <c r="J33" t="n">
         <v>130</v>
       </c>
     </row>
@@ -1444,22 +1539,25 @@
       <c r="C34" t="n">
         <v>3</v>
       </c>
-      <c r="D34" s="4" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="E34" t="n">
+      <c r="D34" t="n">
+        <v>3</v>
+      </c>
+      <c r="E34" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F34" t="n">
         <v>117</v>
       </c>
-      <c r="F34" t="n">
+      <c r="G34" t="n">
         <v>118</v>
       </c>
-      <c r="G34" t="n">
+      <c r="H34" t="n">
         <v>235</v>
       </c>
-      <c r="H34" t="n">
+      <c r="I34" t="n">
         <v>146522</v>
       </c>
-      <c r="I34" t="n">
+      <c r="J34" t="n">
         <v>39</v>
       </c>
     </row>
@@ -1473,24 +1571,27 @@
         <v>6</v>
       </c>
       <c r="C35" t="n">
+        <v>5</v>
+      </c>
+      <c r="D35" t="n">
         <v>4</v>
       </c>
-      <c r="D35" s="4" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="E35" t="n">
-        <v>116</v>
+      <c r="E35" s="4" t="n">
+        <v>0.8</v>
       </c>
       <c r="F35" t="n">
         <v>116</v>
       </c>
       <c r="G35" t="n">
+        <v>116</v>
+      </c>
+      <c r="H35" t="n">
         <v>232</v>
       </c>
-      <c r="H35" t="n">
+      <c r="I35" t="n">
         <v>159650</v>
       </c>
-      <c r="I35" t="n">
+      <c r="J35" t="n">
         <v>29</v>
       </c>
     </row>
@@ -1506,22 +1607,25 @@
       <c r="C36" t="n">
         <v>7</v>
       </c>
-      <c r="D36" s="4" t="n">
+      <c r="D36" t="n">
+        <v>7</v>
+      </c>
+      <c r="E36" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="E36" t="n">
+      <c r="F36" t="n">
         <v>113</v>
       </c>
-      <c r="F36" t="n">
+      <c r="G36" t="n">
         <v>112</v>
       </c>
-      <c r="G36" t="n">
+      <c r="H36" t="n">
         <v>225</v>
       </c>
-      <c r="H36" t="n">
+      <c r="I36" t="n">
         <v>181464</v>
       </c>
-      <c r="I36" t="n">
+      <c r="J36" t="n">
         <v>16</v>
       </c>
     </row>
@@ -1535,24 +1639,27 @@
         <v>9</v>
       </c>
       <c r="C37" t="n">
+        <v>6</v>
+      </c>
+      <c r="D37" t="n">
         <v>4</v>
       </c>
-      <c r="D37" s="4" t="n">
-        <v>0.4444444444444444</v>
-      </c>
-      <c r="E37" t="n">
+      <c r="E37" s="4" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="F37" t="n">
         <v>108</v>
       </c>
-      <c r="F37" t="n">
+      <c r="G37" t="n">
         <v>107</v>
       </c>
-      <c r="G37" t="n">
+      <c r="H37" t="n">
         <v>215</v>
       </c>
-      <c r="H37" t="n">
+      <c r="I37" t="n">
         <v>178315</v>
       </c>
-      <c r="I37" t="n">
+      <c r="J37" t="n">
         <v>27</v>
       </c>
     </row>
@@ -1568,22 +1675,25 @@
       <c r="C38" t="n">
         <v>6</v>
       </c>
-      <c r="D38" s="4" t="n">
-        <v>0.8571428571428571</v>
-      </c>
-      <c r="E38" t="n">
+      <c r="D38" t="n">
+        <v>6</v>
+      </c>
+      <c r="E38" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F38" t="n">
         <v>107</v>
       </c>
-      <c r="F38" t="n">
+      <c r="G38" t="n">
         <v>106</v>
       </c>
-      <c r="G38" t="n">
+      <c r="H38" t="n">
         <v>213</v>
       </c>
-      <c r="H38" t="n">
+      <c r="I38" t="n">
         <v>166891</v>
       </c>
-      <c r="I38" t="n">
+      <c r="J38" t="n">
         <v>18</v>
       </c>
     </row>
@@ -1599,22 +1709,25 @@
       <c r="C39" t="n">
         <v>5</v>
       </c>
-      <c r="D39" s="4" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="E39" t="n">
+      <c r="D39" t="n">
+        <v>5</v>
+      </c>
+      <c r="E39" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F39" t="n">
         <v>106</v>
       </c>
-      <c r="F39" t="n">
+      <c r="G39" t="n">
         <v>104</v>
       </c>
-      <c r="G39" t="n">
+      <c r="H39" t="n">
         <v>210</v>
       </c>
-      <c r="H39" t="n">
+      <c r="I39" t="n">
         <v>149726</v>
       </c>
-      <c r="I39" t="n">
+      <c r="J39" t="n">
         <v>21</v>
       </c>
     </row>
@@ -1628,24 +1741,27 @@
         <v>10</v>
       </c>
       <c r="C40" t="n">
+        <v>5</v>
+      </c>
+      <c r="D40" t="n">
         <v>4</v>
       </c>
-      <c r="D40" s="4" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="E40" t="n">
+      <c r="E40" s="4" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F40" t="n">
         <v>106</v>
       </c>
-      <c r="F40" t="n">
+      <c r="G40" t="n">
         <v>104</v>
       </c>
-      <c r="G40" t="n">
+      <c r="H40" t="n">
         <v>210</v>
       </c>
-      <c r="H40" t="n">
+      <c r="I40" t="n">
         <v>144597</v>
       </c>
-      <c r="I40" t="n">
+      <c r="J40" t="n">
         <v>26</v>
       </c>
     </row>
@@ -1661,22 +1777,25 @@
       <c r="C41" t="n">
         <v>3</v>
       </c>
-      <c r="D41" s="4" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E41" t="n">
+      <c r="D41" t="n">
+        <v>3</v>
+      </c>
+      <c r="E41" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F41" t="n">
         <v>102</v>
       </c>
-      <c r="F41" t="n">
+      <c r="G41" t="n">
         <v>101</v>
       </c>
-      <c r="G41" t="n">
+      <c r="H41" t="n">
         <v>203</v>
       </c>
-      <c r="H41" t="n">
+      <c r="I41" t="n">
         <v>170155</v>
       </c>
-      <c r="I41" t="n">
+      <c r="J41" t="n">
         <v>34</v>
       </c>
     </row>
@@ -1690,24 +1809,27 @@
         <v>7</v>
       </c>
       <c r="C42" t="n">
+        <v>6</v>
+      </c>
+      <c r="D42" t="n">
         <v>5</v>
       </c>
-      <c r="D42" s="4" t="n">
-        <v>0.7142857142857143</v>
-      </c>
-      <c r="E42" t="n">
-        <v>102</v>
+      <c r="E42" s="4" t="n">
+        <v>0.8333333333333334</v>
       </c>
       <c r="F42" t="n">
         <v>102</v>
       </c>
       <c r="G42" t="n">
+        <v>102</v>
+      </c>
+      <c r="H42" t="n">
         <v>204</v>
       </c>
-      <c r="H42" t="n">
+      <c r="I42" t="n">
         <v>119985</v>
       </c>
-      <c r="I42" t="n">
+      <c r="J42" t="n">
         <v>20</v>
       </c>
     </row>
@@ -1723,22 +1845,25 @@
       <c r="C43" t="n">
         <v>3</v>
       </c>
-      <c r="D43" s="4" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="E43" t="n">
+      <c r="D43" t="n">
+        <v>3</v>
+      </c>
+      <c r="E43" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F43" t="n">
         <v>102</v>
       </c>
-      <c r="F43" t="n">
+      <c r="G43" t="n">
         <v>97</v>
       </c>
-      <c r="G43" t="n">
+      <c r="H43" t="n">
         <v>199</v>
       </c>
-      <c r="H43" t="n">
+      <c r="I43" t="n">
         <v>146989</v>
       </c>
-      <c r="I43" t="n">
+      <c r="J43" t="n">
         <v>34</v>
       </c>
     </row>
@@ -1754,22 +1879,25 @@
       <c r="C44" t="n">
         <v>5</v>
       </c>
-      <c r="D44" s="4" t="n">
-        <v>0.8333333333333334</v>
-      </c>
-      <c r="E44" t="n">
+      <c r="D44" t="n">
+        <v>5</v>
+      </c>
+      <c r="E44" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F44" t="n">
         <v>99</v>
       </c>
-      <c r="F44" t="n">
+      <c r="G44" t="n">
         <v>97</v>
       </c>
-      <c r="G44" t="n">
+      <c r="H44" t="n">
         <v>196</v>
       </c>
-      <c r="H44" t="n">
+      <c r="I44" t="n">
         <v>134932</v>
       </c>
-      <c r="I44" t="n">
+      <c r="J44" t="n">
         <v>20</v>
       </c>
     </row>
@@ -1783,24 +1911,27 @@
         <v>2</v>
       </c>
       <c r="C45" t="n">
+        <v>2</v>
+      </c>
+      <c r="D45" t="n">
         <v>1</v>
       </c>
-      <c r="D45" s="4" t="n">
+      <c r="E45" s="4" t="n">
         <v>0.5</v>
       </c>
-      <c r="E45" t="n">
+      <c r="F45" t="n">
         <v>99</v>
       </c>
-      <c r="F45" t="n">
+      <c r="G45" t="n">
         <v>98</v>
       </c>
-      <c r="G45" t="n">
+      <c r="H45" t="n">
         <v>197</v>
       </c>
-      <c r="H45" t="n">
+      <c r="I45" t="n">
         <v>178741</v>
       </c>
-      <c r="I45" t="n">
+      <c r="J45" t="n">
         <v>99</v>
       </c>
     </row>
@@ -1816,22 +1947,25 @@
       <c r="C46" t="n">
         <v>4</v>
       </c>
-      <c r="D46" s="4" t="n">
-        <v>0.5714285714285714</v>
-      </c>
-      <c r="E46" t="n">
+      <c r="D46" t="n">
+        <v>4</v>
+      </c>
+      <c r="E46" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F46" t="n">
         <v>96</v>
       </c>
-      <c r="F46" t="n">
+      <c r="G46" t="n">
         <v>95</v>
       </c>
-      <c r="G46" t="n">
+      <c r="H46" t="n">
         <v>191</v>
       </c>
-      <c r="H46" t="n">
+      <c r="I46" t="n">
         <v>151027</v>
       </c>
-      <c r="I46" t="n">
+      <c r="J46" t="n">
         <v>24</v>
       </c>
     </row>
@@ -1845,24 +1979,27 @@
         <v>8</v>
       </c>
       <c r="C47" t="n">
+        <v>6</v>
+      </c>
+      <c r="D47" t="n">
         <v>4</v>
       </c>
-      <c r="D47" s="4" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E47" t="n">
+      <c r="E47" s="4" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="F47" t="n">
         <v>95</v>
       </c>
-      <c r="F47" t="n">
+      <c r="G47" t="n">
         <v>93</v>
       </c>
-      <c r="G47" t="n">
+      <c r="H47" t="n">
         <v>188</v>
       </c>
-      <c r="H47" t="n">
+      <c r="I47" t="n">
         <v>129166</v>
       </c>
-      <c r="I47" t="n">
+      <c r="J47" t="n">
         <v>24</v>
       </c>
     </row>
@@ -1876,24 +2013,27 @@
         <v>12</v>
       </c>
       <c r="C48" t="n">
+        <v>7</v>
+      </c>
+      <c r="D48" t="n">
         <v>6</v>
       </c>
-      <c r="D48" s="4" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E48" t="n">
+      <c r="E48" s="4" t="n">
+        <v>0.8571428571428571</v>
+      </c>
+      <c r="F48" t="n">
         <v>93</v>
       </c>
-      <c r="F48" t="n">
+      <c r="G48" t="n">
         <v>90</v>
       </c>
-      <c r="G48" t="n">
+      <c r="H48" t="n">
         <v>183</v>
       </c>
-      <c r="H48" t="n">
+      <c r="I48" t="n">
         <v>130292</v>
       </c>
-      <c r="I48" t="n">
+      <c r="J48" t="n">
         <v>16</v>
       </c>
     </row>
@@ -1907,24 +2047,27 @@
         <v>11</v>
       </c>
       <c r="C49" t="n">
+        <v>8</v>
+      </c>
+      <c r="D49" t="n">
         <v>7</v>
       </c>
-      <c r="D49" s="4" t="n">
-        <v>0.6363636363636364</v>
-      </c>
-      <c r="E49" t="n">
-        <v>92</v>
+      <c r="E49" s="4" t="n">
+        <v>0.875</v>
       </c>
       <c r="F49" t="n">
         <v>92</v>
       </c>
       <c r="G49" t="n">
+        <v>92</v>
+      </c>
+      <c r="H49" t="n">
         <v>184</v>
       </c>
-      <c r="H49" t="n">
+      <c r="I49" t="n">
         <v>133496</v>
       </c>
-      <c r="I49" t="n">
+      <c r="J49" t="n">
         <v>13</v>
       </c>
     </row>
@@ -1940,22 +2083,25 @@
       <c r="C50" t="n">
         <v>6</v>
       </c>
-      <c r="D50" s="4" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="E50" t="n">
+      <c r="D50" t="n">
+        <v>6</v>
+      </c>
+      <c r="E50" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F50" t="n">
         <v>91</v>
       </c>
-      <c r="F50" t="n">
+      <c r="G50" t="n">
         <v>89</v>
       </c>
-      <c r="G50" t="n">
+      <c r="H50" t="n">
         <v>180</v>
       </c>
-      <c r="H50" t="n">
+      <c r="I50" t="n">
         <v>134223</v>
       </c>
-      <c r="I50" t="n">
+      <c r="J50" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1969,24 +2115,27 @@
         <v>6</v>
       </c>
       <c r="C51" t="n">
+        <v>6</v>
+      </c>
+      <c r="D51" t="n">
         <v>5</v>
       </c>
-      <c r="D51" s="4" t="n">
+      <c r="E51" s="4" t="n">
         <v>0.8333333333333334</v>
-      </c>
-      <c r="E51" t="n">
-        <v>86</v>
       </c>
       <c r="F51" t="n">
         <v>86</v>
       </c>
       <c r="G51" t="n">
+        <v>86</v>
+      </c>
+      <c r="H51" t="n">
         <v>172</v>
       </c>
-      <c r="H51" t="n">
+      <c r="I51" t="n">
         <v>126152</v>
       </c>
-      <c r="I51" t="n">
+      <c r="J51" t="n">
         <v>17</v>
       </c>
     </row>
@@ -2000,24 +2149,27 @@
         <v>3</v>
       </c>
       <c r="C52" t="n">
+        <v>3</v>
+      </c>
+      <c r="D52" t="n">
         <v>2</v>
       </c>
-      <c r="D52" s="4" t="n">
+      <c r="E52" s="4" t="n">
         <v>0.6666666666666666</v>
       </c>
-      <c r="E52" t="n">
+      <c r="F52" t="n">
         <v>85</v>
       </c>
-      <c r="F52" t="n">
+      <c r="G52" t="n">
         <v>84</v>
       </c>
-      <c r="G52" t="n">
+      <c r="H52" t="n">
         <v>169</v>
       </c>
-      <c r="H52" t="n">
+      <c r="I52" t="n">
         <v>94654</v>
       </c>
-      <c r="I52" t="n">
+      <c r="J52" t="n">
         <v>42</v>
       </c>
     </row>
@@ -2033,22 +2185,25 @@
       <c r="C53" t="n">
         <v>6</v>
       </c>
-      <c r="D53" s="4" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="E53" t="n">
+      <c r="D53" t="n">
+        <v>6</v>
+      </c>
+      <c r="E53" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F53" t="n">
         <v>82</v>
       </c>
-      <c r="F53" t="n">
+      <c r="G53" t="n">
         <v>79</v>
       </c>
-      <c r="G53" t="n">
+      <c r="H53" t="n">
         <v>161</v>
       </c>
-      <c r="H53" t="n">
+      <c r="I53" t="n">
         <v>119272</v>
       </c>
-      <c r="I53" t="n">
+      <c r="J53" t="n">
         <v>14</v>
       </c>
     </row>
@@ -2064,22 +2219,25 @@
       <c r="C54" t="n">
         <v>2</v>
       </c>
-      <c r="D54" s="4" t="n">
+      <c r="D54" t="n">
+        <v>2</v>
+      </c>
+      <c r="E54" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="E54" t="n">
+      <c r="F54" t="n">
         <v>82</v>
       </c>
-      <c r="F54" t="n">
+      <c r="G54" t="n">
         <v>80</v>
       </c>
-      <c r="G54" t="n">
+      <c r="H54" t="n">
         <v>162</v>
       </c>
-      <c r="H54" t="n">
+      <c r="I54" t="n">
         <v>140602</v>
       </c>
-      <c r="I54" t="n">
+      <c r="J54" t="n">
         <v>41</v>
       </c>
     </row>
@@ -2095,22 +2253,25 @@
       <c r="C55" t="n">
         <v>4</v>
       </c>
-      <c r="D55" s="4" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="E55" t="n">
+      <c r="D55" t="n">
+        <v>4</v>
+      </c>
+      <c r="E55" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F55" t="n">
         <v>80</v>
       </c>
-      <c r="F55" t="n">
+      <c r="G55" t="n">
         <v>81</v>
       </c>
-      <c r="G55" t="n">
+      <c r="H55" t="n">
         <v>161</v>
       </c>
-      <c r="H55" t="n">
+      <c r="I55" t="n">
         <v>118914</v>
       </c>
-      <c r="I55" t="n">
+      <c r="J55" t="n">
         <v>20</v>
       </c>
     </row>
@@ -2126,22 +2287,25 @@
       <c r="C56" t="n">
         <v>3</v>
       </c>
-      <c r="D56" s="4" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E56" t="n">
+      <c r="D56" t="n">
+        <v>3</v>
+      </c>
+      <c r="E56" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F56" t="n">
         <v>79</v>
       </c>
-      <c r="F56" t="n">
+      <c r="G56" t="n">
         <v>77</v>
       </c>
-      <c r="G56" t="n">
+      <c r="H56" t="n">
         <v>156</v>
       </c>
-      <c r="H56" t="n">
+      <c r="I56" t="n">
         <v>102286</v>
       </c>
-      <c r="I56" t="n">
+      <c r="J56" t="n">
         <v>26</v>
       </c>
     </row>
@@ -2155,24 +2319,27 @@
         <v>8</v>
       </c>
       <c r="C57" t="n">
+        <v>6</v>
+      </c>
+      <c r="D57" t="n">
         <v>5</v>
       </c>
-      <c r="D57" s="4" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="E57" t="n">
-        <v>79</v>
+      <c r="E57" s="4" t="n">
+        <v>0.8333333333333334</v>
       </c>
       <c r="F57" t="n">
         <v>79</v>
       </c>
       <c r="G57" t="n">
+        <v>79</v>
+      </c>
+      <c r="H57" t="n">
         <v>158</v>
       </c>
-      <c r="H57" t="n">
+      <c r="I57" t="n">
         <v>125691</v>
       </c>
-      <c r="I57" t="n">
+      <c r="J57" t="n">
         <v>16</v>
       </c>
     </row>
@@ -2186,24 +2353,27 @@
         <v>9</v>
       </c>
       <c r="C58" t="n">
+        <v>8</v>
+      </c>
+      <c r="D58" t="n">
         <v>4</v>
       </c>
-      <c r="D58" s="4" t="n">
-        <v>0.4444444444444444</v>
-      </c>
-      <c r="E58" t="n">
-        <v>74</v>
+      <c r="E58" s="4" t="n">
+        <v>0.5</v>
       </c>
       <c r="F58" t="n">
         <v>74</v>
       </c>
       <c r="G58" t="n">
+        <v>74</v>
+      </c>
+      <c r="H58" t="n">
         <v>148</v>
       </c>
-      <c r="H58" t="n">
+      <c r="I58" t="n">
         <v>108160</v>
       </c>
-      <c r="I58" t="n">
+      <c r="J58" t="n">
         <v>18</v>
       </c>
     </row>
@@ -2219,22 +2389,25 @@
       <c r="C59" t="n">
         <v>2</v>
       </c>
-      <c r="D59" s="4" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E59" t="n">
+      <c r="D59" t="n">
+        <v>2</v>
+      </c>
+      <c r="E59" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F59" t="n">
         <v>73</v>
       </c>
-      <c r="F59" t="n">
+      <c r="G59" t="n">
         <v>72</v>
       </c>
-      <c r="G59" t="n">
+      <c r="H59" t="n">
         <v>145</v>
       </c>
-      <c r="H59" t="n">
+      <c r="I59" t="n">
         <v>98484</v>
       </c>
-      <c r="I59" t="n">
+      <c r="J59" t="n">
         <v>36</v>
       </c>
     </row>
@@ -2248,24 +2421,27 @@
         <v>8</v>
       </c>
       <c r="C60" t="n">
+        <v>4</v>
+      </c>
+      <c r="D60" t="n">
         <v>2</v>
       </c>
-      <c r="D60" s="4" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="E60" t="n">
+      <c r="E60" s="4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F60" t="n">
         <v>70</v>
       </c>
-      <c r="F60" t="n">
+      <c r="G60" t="n">
         <v>69</v>
       </c>
-      <c r="G60" t="n">
+      <c r="H60" t="n">
         <v>139</v>
       </c>
-      <c r="H60" t="n">
+      <c r="I60" t="n">
         <v>88769</v>
       </c>
-      <c r="I60" t="n">
+      <c r="J60" t="n">
         <v>35</v>
       </c>
     </row>
@@ -2281,22 +2457,25 @@
       <c r="C61" t="n">
         <v>3</v>
       </c>
-      <c r="D61" s="4" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E61" t="n">
-        <v>67</v>
+      <c r="D61" t="n">
+        <v>3</v>
+      </c>
+      <c r="E61" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="F61" t="n">
         <v>67</v>
       </c>
       <c r="G61" t="n">
+        <v>67</v>
+      </c>
+      <c r="H61" t="n">
         <v>134</v>
       </c>
-      <c r="H61" t="n">
+      <c r="I61" t="n">
         <v>93382</v>
       </c>
-      <c r="I61" t="n">
+      <c r="J61" t="n">
         <v>22</v>
       </c>
     </row>
@@ -2310,24 +2489,27 @@
         <v>8</v>
       </c>
       <c r="C62" t="n">
+        <v>6</v>
+      </c>
+      <c r="D62" t="n">
         <v>5</v>
       </c>
-      <c r="D62" s="4" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="E62" t="n">
-        <v>64</v>
+      <c r="E62" s="4" t="n">
+        <v>0.8333333333333334</v>
       </c>
       <c r="F62" t="n">
         <v>64</v>
       </c>
       <c r="G62" t="n">
+        <v>64</v>
+      </c>
+      <c r="H62" t="n">
         <v>128</v>
       </c>
-      <c r="H62" t="n">
+      <c r="I62" t="n">
         <v>89894</v>
       </c>
-      <c r="I62" t="n">
+      <c r="J62" t="n">
         <v>13</v>
       </c>
     </row>
@@ -2341,24 +2523,27 @@
         <v>7</v>
       </c>
       <c r="C63" t="n">
+        <v>4</v>
+      </c>
+      <c r="D63" t="n">
         <v>3</v>
       </c>
-      <c r="D63" s="4" t="n">
-        <v>0.4285714285714285</v>
-      </c>
-      <c r="E63" t="n">
-        <v>63</v>
+      <c r="E63" s="4" t="n">
+        <v>0.75</v>
       </c>
       <c r="F63" t="n">
         <v>63</v>
       </c>
       <c r="G63" t="n">
+        <v>63</v>
+      </c>
+      <c r="H63" t="n">
         <v>126</v>
       </c>
-      <c r="H63" t="n">
+      <c r="I63" t="n">
         <v>108299</v>
       </c>
-      <c r="I63" t="n">
+      <c r="J63" t="n">
         <v>21</v>
       </c>
     </row>
@@ -2374,22 +2559,25 @@
       <c r="C64" t="n">
         <v>1</v>
       </c>
-      <c r="D64" s="4" t="n">
+      <c r="D64" t="n">
         <v>1</v>
       </c>
-      <c r="E64" t="n">
-        <v>62</v>
+      <c r="E64" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="F64" t="n">
         <v>62</v>
       </c>
       <c r="G64" t="n">
+        <v>62</v>
+      </c>
+      <c r="H64" t="n">
         <v>124</v>
       </c>
-      <c r="H64" t="n">
+      <c r="I64" t="n">
         <v>138594</v>
       </c>
-      <c r="I64" t="n">
+      <c r="J64" t="n">
         <v>62</v>
       </c>
     </row>
@@ -2403,24 +2591,27 @@
         <v>14</v>
       </c>
       <c r="C65" t="n">
+        <v>6</v>
+      </c>
+      <c r="D65" t="n">
         <v>5</v>
       </c>
-      <c r="D65" s="4" t="n">
-        <v>0.3571428571428572</v>
-      </c>
-      <c r="E65" t="n">
+      <c r="E65" s="4" t="n">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="F65" t="n">
         <v>61</v>
       </c>
-      <c r="F65" t="n">
+      <c r="G65" t="n">
         <v>62</v>
       </c>
-      <c r="G65" t="n">
+      <c r="H65" t="n">
         <v>123</v>
       </c>
-      <c r="H65" t="n">
+      <c r="I65" t="n">
         <v>92974</v>
       </c>
-      <c r="I65" t="n">
+      <c r="J65" t="n">
         <v>12</v>
       </c>
     </row>
@@ -2436,22 +2627,25 @@
       <c r="C66" t="n">
         <v>2</v>
       </c>
-      <c r="D66" s="4" t="n">
+      <c r="D66" t="n">
+        <v>2</v>
+      </c>
+      <c r="E66" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="E66" t="n">
+      <c r="F66" t="n">
         <v>60</v>
       </c>
-      <c r="F66" t="n">
+      <c r="G66" t="n">
         <v>59</v>
       </c>
-      <c r="G66" t="n">
+      <c r="H66" t="n">
         <v>119</v>
       </c>
-      <c r="H66" t="n">
+      <c r="I66" t="n">
         <v>103077</v>
       </c>
-      <c r="I66" t="n">
+      <c r="J66" t="n">
         <v>30</v>
       </c>
     </row>
@@ -2467,22 +2661,25 @@
       <c r="C67" t="n">
         <v>2</v>
       </c>
-      <c r="D67" s="4" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="E67" t="n">
+      <c r="D67" t="n">
+        <v>2</v>
+      </c>
+      <c r="E67" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F67" t="n">
         <v>60</v>
       </c>
-      <c r="F67" t="n">
+      <c r="G67" t="n">
         <v>59</v>
       </c>
-      <c r="G67" t="n">
+      <c r="H67" t="n">
         <v>119</v>
       </c>
-      <c r="H67" t="n">
+      <c r="I67" t="n">
         <v>96131</v>
       </c>
-      <c r="I67" t="n">
+      <c r="J67" t="n">
         <v>30</v>
       </c>
     </row>
@@ -2498,22 +2695,25 @@
       <c r="C68" t="n">
         <v>3</v>
       </c>
-      <c r="D68" s="4" t="n">
+      <c r="D68" t="n">
+        <v>3</v>
+      </c>
+      <c r="E68" s="4" t="n">
         <v>1</v>
-      </c>
-      <c r="E68" t="n">
-        <v>59</v>
       </c>
       <c r="F68" t="n">
         <v>59</v>
       </c>
       <c r="G68" t="n">
+        <v>59</v>
+      </c>
+      <c r="H68" t="n">
         <v>118</v>
       </c>
-      <c r="H68" t="n">
+      <c r="I68" t="n">
         <v>99106</v>
       </c>
-      <c r="I68" t="n">
+      <c r="J68" t="n">
         <v>20</v>
       </c>
     </row>
@@ -2529,22 +2729,25 @@
       <c r="C69" t="n">
         <v>5</v>
       </c>
-      <c r="D69" s="4" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="E69" t="n">
-        <v>58</v>
+      <c r="D69" t="n">
+        <v>5</v>
+      </c>
+      <c r="E69" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="F69" t="n">
         <v>58</v>
       </c>
       <c r="G69" t="n">
+        <v>58</v>
+      </c>
+      <c r="H69" t="n">
         <v>116</v>
       </c>
-      <c r="H69" t="n">
+      <c r="I69" t="n">
         <v>78484</v>
       </c>
-      <c r="I69" t="n">
+      <c r="J69" t="n">
         <v>12</v>
       </c>
     </row>
@@ -2560,22 +2763,25 @@
       <c r="C70" t="n">
         <v>1</v>
       </c>
-      <c r="D70" s="4" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E70" t="n">
+      <c r="D70" t="n">
+        <v>1</v>
+      </c>
+      <c r="E70" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F70" t="n">
         <v>57</v>
       </c>
-      <c r="F70" t="n">
+      <c r="G70" t="n">
         <v>56</v>
       </c>
-      <c r="G70" t="n">
+      <c r="H70" t="n">
         <v>113</v>
       </c>
-      <c r="H70" t="n">
+      <c r="I70" t="n">
         <v>76180</v>
       </c>
-      <c r="I70" t="n">
+      <c r="J70" t="n">
         <v>57</v>
       </c>
     </row>
@@ -2589,24 +2795,27 @@
         <v>3</v>
       </c>
       <c r="C71" t="n">
+        <v>2</v>
+      </c>
+      <c r="D71" t="n">
         <v>1</v>
       </c>
-      <c r="D71" s="4" t="n">
-        <v>0.3333333333333333</v>
-      </c>
-      <c r="E71" t="n">
+      <c r="E71" s="4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F71" t="n">
         <v>56</v>
       </c>
-      <c r="F71" t="n">
+      <c r="G71" t="n">
         <v>55</v>
       </c>
-      <c r="G71" t="n">
+      <c r="H71" t="n">
         <v>111</v>
       </c>
-      <c r="H71" t="n">
+      <c r="I71" t="n">
         <v>94572</v>
       </c>
-      <c r="I71" t="n">
+      <c r="J71" t="n">
         <v>56</v>
       </c>
     </row>
@@ -2620,24 +2829,27 @@
         <v>10</v>
       </c>
       <c r="C72" t="n">
+        <v>6</v>
+      </c>
+      <c r="D72" t="n">
         <v>4</v>
       </c>
-      <c r="D72" s="4" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="E72" t="n">
-        <v>56</v>
+      <c r="E72" s="4" t="n">
+        <v>0.6666666666666666</v>
       </c>
       <c r="F72" t="n">
         <v>56</v>
       </c>
       <c r="G72" t="n">
+        <v>56</v>
+      </c>
+      <c r="H72" t="n">
         <v>112</v>
       </c>
-      <c r="H72" t="n">
+      <c r="I72" t="n">
         <v>72581</v>
       </c>
-      <c r="I72" t="n">
+      <c r="J72" t="n">
         <v>14</v>
       </c>
     </row>
@@ -2651,24 +2863,27 @@
         <v>8</v>
       </c>
       <c r="C73" t="n">
+        <v>6</v>
+      </c>
+      <c r="D73" t="n">
         <v>3</v>
       </c>
-      <c r="D73" s="4" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="E73" t="n">
-        <v>55</v>
+      <c r="E73" s="4" t="n">
+        <v>0.5</v>
       </c>
       <c r="F73" t="n">
         <v>55</v>
       </c>
       <c r="G73" t="n">
+        <v>55</v>
+      </c>
+      <c r="H73" t="n">
         <v>110</v>
       </c>
-      <c r="H73" t="n">
+      <c r="I73" t="n">
         <v>81861</v>
       </c>
-      <c r="I73" t="n">
+      <c r="J73" t="n">
         <v>18</v>
       </c>
     </row>
@@ -2682,24 +2897,27 @@
         <v>12</v>
       </c>
       <c r="C74" t="n">
+        <v>10</v>
+      </c>
+      <c r="D74" t="n">
         <v>8</v>
       </c>
-      <c r="D74" s="4" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="E74" t="n">
+      <c r="E74" s="4" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F74" t="n">
         <v>55</v>
       </c>
-      <c r="F74" t="n">
+      <c r="G74" t="n">
         <v>53</v>
       </c>
-      <c r="G74" t="n">
+      <c r="H74" t="n">
         <v>108</v>
       </c>
-      <c r="H74" t="n">
+      <c r="I74" t="n">
         <v>54378</v>
       </c>
-      <c r="I74" t="n">
+      <c r="J74" t="n">
         <v>7</v>
       </c>
     </row>
@@ -2715,22 +2933,25 @@
       <c r="C75" t="n">
         <v>1</v>
       </c>
-      <c r="D75" s="4" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E75" t="n">
-        <v>55</v>
+      <c r="D75" t="n">
+        <v>1</v>
+      </c>
+      <c r="E75" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="F75" t="n">
         <v>55</v>
       </c>
       <c r="G75" t="n">
+        <v>55</v>
+      </c>
+      <c r="H75" t="n">
         <v>110</v>
       </c>
-      <c r="H75" t="n">
+      <c r="I75" t="n">
         <v>105930</v>
       </c>
-      <c r="I75" t="n">
+      <c r="J75" t="n">
         <v>55</v>
       </c>
     </row>
@@ -2746,22 +2967,25 @@
       <c r="C76" t="n">
         <v>5</v>
       </c>
-      <c r="D76" s="4" t="n">
-        <v>0.2631578947368421</v>
-      </c>
-      <c r="E76" t="n">
+      <c r="D76" t="n">
+        <v>5</v>
+      </c>
+      <c r="E76" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F76" t="n">
         <v>53</v>
       </c>
-      <c r="F76" t="n">
+      <c r="G76" t="n">
         <v>52</v>
       </c>
-      <c r="G76" t="n">
+      <c r="H76" t="n">
         <v>105</v>
       </c>
-      <c r="H76" t="n">
+      <c r="I76" t="n">
         <v>66548</v>
       </c>
-      <c r="I76" t="n">
+      <c r="J76" t="n">
         <v>11</v>
       </c>
     </row>
@@ -2777,22 +3001,25 @@
       <c r="C77" t="n">
         <v>3</v>
       </c>
-      <c r="D77" s="4" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="E77" t="n">
-        <v>51</v>
+      <c r="D77" t="n">
+        <v>3</v>
+      </c>
+      <c r="E77" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="F77" t="n">
         <v>51</v>
       </c>
       <c r="G77" t="n">
+        <v>51</v>
+      </c>
+      <c r="H77" t="n">
         <v>102</v>
       </c>
-      <c r="H77" t="n">
+      <c r="I77" t="n">
         <v>69866</v>
       </c>
-      <c r="I77" t="n">
+      <c r="J77" t="n">
         <v>17</v>
       </c>
     </row>
@@ -2806,24 +3033,27 @@
         <v>2</v>
       </c>
       <c r="C78" t="n">
+        <v>2</v>
+      </c>
+      <c r="D78" t="n">
         <v>1</v>
       </c>
-      <c r="D78" s="4" t="n">
+      <c r="E78" s="4" t="n">
         <v>0.5</v>
-      </c>
-      <c r="E78" t="n">
-        <v>49</v>
       </c>
       <c r="F78" t="n">
         <v>49</v>
       </c>
       <c r="G78" t="n">
+        <v>49</v>
+      </c>
+      <c r="H78" t="n">
         <v>98</v>
       </c>
-      <c r="H78" t="n">
+      <c r="I78" t="n">
         <v>81259</v>
       </c>
-      <c r="I78" t="n">
+      <c r="J78" t="n">
         <v>49</v>
       </c>
     </row>
@@ -2839,22 +3069,25 @@
       <c r="C79" t="n">
         <v>2</v>
       </c>
-      <c r="D79" s="4" t="n">
+      <c r="D79" t="n">
+        <v>2</v>
+      </c>
+      <c r="E79" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="E79" t="n">
+      <c r="F79" t="n">
         <v>47</v>
       </c>
-      <c r="F79" t="n">
+      <c r="G79" t="n">
         <v>46</v>
       </c>
-      <c r="G79" t="n">
+      <c r="H79" t="n">
         <v>93</v>
       </c>
-      <c r="H79" t="n">
+      <c r="I79" t="n">
         <v>62930</v>
       </c>
-      <c r="I79" t="n">
+      <c r="J79" t="n">
         <v>24</v>
       </c>
     </row>
@@ -2868,24 +3101,27 @@
         <v>11</v>
       </c>
       <c r="C80" t="n">
+        <v>7</v>
+      </c>
+      <c r="D80" t="n">
         <v>5</v>
       </c>
-      <c r="D80" s="4" t="n">
-        <v>0.4545454545454545</v>
-      </c>
-      <c r="E80" t="n">
+      <c r="E80" s="4" t="n">
+        <v>0.7142857142857143</v>
+      </c>
+      <c r="F80" t="n">
         <v>45</v>
       </c>
-      <c r="F80" t="n">
+      <c r="G80" t="n">
         <v>43</v>
       </c>
-      <c r="G80" t="n">
+      <c r="H80" t="n">
         <v>88</v>
       </c>
-      <c r="H80" t="n">
+      <c r="I80" t="n">
         <v>58040</v>
       </c>
-      <c r="I80" t="n">
+      <c r="J80" t="n">
         <v>9</v>
       </c>
     </row>
@@ -2901,22 +3137,25 @@
       <c r="C81" t="n">
         <v>2</v>
       </c>
-      <c r="D81" s="4" t="n">
+      <c r="D81" t="n">
+        <v>2</v>
+      </c>
+      <c r="E81" s="4" t="n">
         <v>1</v>
-      </c>
-      <c r="E81" t="n">
-        <v>45</v>
       </c>
       <c r="F81" t="n">
         <v>45</v>
       </c>
       <c r="G81" t="n">
+        <v>45</v>
+      </c>
+      <c r="H81" t="n">
         <v>90</v>
       </c>
-      <c r="H81" t="n">
+      <c r="I81" t="n">
         <v>65340</v>
       </c>
-      <c r="I81" t="n">
+      <c r="J81" t="n">
         <v>22</v>
       </c>
     </row>
@@ -2932,22 +3171,25 @@
       <c r="C82" t="n">
         <v>1</v>
       </c>
-      <c r="D82" s="4" t="n">
-        <v>0.3333333333333333</v>
-      </c>
-      <c r="E82" t="n">
+      <c r="D82" t="n">
+        <v>1</v>
+      </c>
+      <c r="E82" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F82" t="n">
         <v>44</v>
       </c>
-      <c r="F82" t="n">
+      <c r="G82" t="n">
         <v>43</v>
       </c>
-      <c r="G82" t="n">
+      <c r="H82" t="n">
         <v>87</v>
       </c>
-      <c r="H82" t="n">
+      <c r="I82" t="n">
         <v>60697</v>
       </c>
-      <c r="I82" t="n">
+      <c r="J82" t="n">
         <v>44</v>
       </c>
     </row>
@@ -2963,22 +3205,25 @@
       <c r="C83" t="n">
         <v>3</v>
       </c>
-      <c r="D83" s="4" t="n">
+      <c r="D83" t="n">
+        <v>3</v>
+      </c>
+      <c r="E83" s="4" t="n">
         <v>1</v>
-      </c>
-      <c r="E83" t="n">
-        <v>43</v>
       </c>
       <c r="F83" t="n">
         <v>43</v>
       </c>
       <c r="G83" t="n">
+        <v>43</v>
+      </c>
+      <c r="H83" t="n">
         <v>86</v>
       </c>
-      <c r="H83" t="n">
+      <c r="I83" t="n">
         <v>54824</v>
       </c>
-      <c r="I83" t="n">
+      <c r="J83" t="n">
         <v>14</v>
       </c>
     </row>
@@ -2992,24 +3237,27 @@
         <v>3</v>
       </c>
       <c r="C84" t="n">
+        <v>2</v>
+      </c>
+      <c r="D84" t="n">
         <v>1</v>
       </c>
-      <c r="D84" s="4" t="n">
-        <v>0.3333333333333333</v>
-      </c>
-      <c r="E84" t="n">
-        <v>42</v>
+      <c r="E84" s="4" t="n">
+        <v>0.5</v>
       </c>
       <c r="F84" t="n">
         <v>42</v>
       </c>
       <c r="G84" t="n">
+        <v>42</v>
+      </c>
+      <c r="H84" t="n">
         <v>84</v>
       </c>
-      <c r="H84" t="n">
+      <c r="I84" t="n">
         <v>60833</v>
       </c>
-      <c r="I84" t="n">
+      <c r="J84" t="n">
         <v>42</v>
       </c>
     </row>
@@ -3025,22 +3273,25 @@
       <c r="C85" t="n">
         <v>3</v>
       </c>
-      <c r="D85" s="4" t="n">
+      <c r="D85" t="n">
+        <v>3</v>
+      </c>
+      <c r="E85" s="4" t="n">
         <v>1</v>
-      </c>
-      <c r="E85" t="n">
-        <v>39</v>
       </c>
       <c r="F85" t="n">
         <v>39</v>
       </c>
       <c r="G85" t="n">
+        <v>39</v>
+      </c>
+      <c r="H85" t="n">
         <v>78</v>
       </c>
-      <c r="H85" t="n">
+      <c r="I85" t="n">
         <v>54875</v>
       </c>
-      <c r="I85" t="n">
+      <c r="J85" t="n">
         <v>13</v>
       </c>
     </row>
@@ -3056,22 +3307,25 @@
       <c r="C86" t="n">
         <v>2</v>
       </c>
-      <c r="D86" s="4" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E86" t="n">
-        <v>37</v>
+      <c r="D86" t="n">
+        <v>2</v>
+      </c>
+      <c r="E86" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="F86" t="n">
         <v>37</v>
       </c>
       <c r="G86" t="n">
+        <v>37</v>
+      </c>
+      <c r="H86" t="n">
         <v>74</v>
       </c>
-      <c r="H86" t="n">
+      <c r="I86" t="n">
         <v>45424</v>
       </c>
-      <c r="I86" t="n">
+      <c r="J86" t="n">
         <v>18</v>
       </c>
     </row>
@@ -3087,22 +3341,25 @@
       <c r="C87" t="n">
         <v>1</v>
       </c>
-      <c r="D87" s="4" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="E87" t="n">
+      <c r="D87" t="n">
+        <v>1</v>
+      </c>
+      <c r="E87" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F87" t="n">
         <v>37</v>
       </c>
-      <c r="F87" t="n">
+      <c r="G87" t="n">
         <v>36</v>
       </c>
-      <c r="G87" t="n">
+      <c r="H87" t="n">
         <v>73</v>
       </c>
-      <c r="H87" t="n">
+      <c r="I87" t="n">
         <v>41549</v>
       </c>
-      <c r="I87" t="n">
+      <c r="J87" t="n">
         <v>37</v>
       </c>
     </row>
@@ -3118,22 +3375,25 @@
       <c r="C88" t="n">
         <v>2</v>
       </c>
-      <c r="D88" s="4" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="E88" t="n">
-        <v>36</v>
+      <c r="D88" t="n">
+        <v>2</v>
+      </c>
+      <c r="E88" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="F88" t="n">
         <v>36</v>
       </c>
       <c r="G88" t="n">
+        <v>36</v>
+      </c>
+      <c r="H88" t="n">
         <v>72</v>
       </c>
-      <c r="H88" t="n">
+      <c r="I88" t="n">
         <v>36412</v>
       </c>
-      <c r="I88" t="n">
+      <c r="J88" t="n">
         <v>18</v>
       </c>
     </row>
@@ -3149,22 +3409,25 @@
       <c r="C89" t="n">
         <v>1</v>
       </c>
-      <c r="D89" s="4" t="n">
-        <v>0.3333333333333333</v>
-      </c>
-      <c r="E89" t="n">
-        <v>34</v>
+      <c r="D89" t="n">
+        <v>1</v>
+      </c>
+      <c r="E89" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="F89" t="n">
         <v>34</v>
       </c>
       <c r="G89" t="n">
+        <v>34</v>
+      </c>
+      <c r="H89" t="n">
         <v>68</v>
       </c>
-      <c r="H89" t="n">
+      <c r="I89" t="n">
         <v>58216</v>
       </c>
-      <c r="I89" t="n">
+      <c r="J89" t="n">
         <v>34</v>
       </c>
     </row>
@@ -3180,22 +3443,25 @@
       <c r="C90" t="n">
         <v>2</v>
       </c>
-      <c r="D90" s="4" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E90" t="n">
-        <v>33</v>
+      <c r="D90" t="n">
+        <v>2</v>
+      </c>
+      <c r="E90" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="F90" t="n">
         <v>33</v>
       </c>
       <c r="G90" t="n">
+        <v>33</v>
+      </c>
+      <c r="H90" t="n">
         <v>66</v>
       </c>
-      <c r="H90" t="n">
+      <c r="I90" t="n">
         <v>39823</v>
       </c>
-      <c r="I90" t="n">
+      <c r="J90" t="n">
         <v>16</v>
       </c>
     </row>
@@ -3211,22 +3477,25 @@
       <c r="C91" t="n">
         <v>4</v>
       </c>
-      <c r="D91" s="4" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="E91" t="n">
-        <v>33</v>
+      <c r="D91" t="n">
+        <v>4</v>
+      </c>
+      <c r="E91" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="F91" t="n">
         <v>33</v>
       </c>
       <c r="G91" t="n">
+        <v>33</v>
+      </c>
+      <c r="H91" t="n">
         <v>66</v>
       </c>
-      <c r="H91" t="n">
+      <c r="I91" t="n">
         <v>51998</v>
       </c>
-      <c r="I91" t="n">
+      <c r="J91" t="n">
         <v>8</v>
       </c>
     </row>
@@ -3242,22 +3511,25 @@
       <c r="C92" t="n">
         <v>3</v>
       </c>
-      <c r="D92" s="4" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="E92" t="n">
+      <c r="D92" t="n">
+        <v>3</v>
+      </c>
+      <c r="E92" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F92" t="n">
         <v>33</v>
       </c>
-      <c r="F92" t="n">
+      <c r="G92" t="n">
         <v>32</v>
       </c>
-      <c r="G92" t="n">
+      <c r="H92" t="n">
         <v>65</v>
       </c>
-      <c r="H92" t="n">
+      <c r="I92" t="n">
         <v>41309</v>
       </c>
-      <c r="I92" t="n">
+      <c r="J92" t="n">
         <v>11</v>
       </c>
     </row>
@@ -3273,22 +3545,25 @@
       <c r="C93" t="n">
         <v>3</v>
       </c>
-      <c r="D93" s="4" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="E93" t="n">
+      <c r="D93" t="n">
+        <v>3</v>
+      </c>
+      <c r="E93" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F93" t="n">
         <v>32</v>
       </c>
-      <c r="F93" t="n">
+      <c r="G93" t="n">
         <v>31</v>
       </c>
-      <c r="G93" t="n">
+      <c r="H93" t="n">
         <v>63</v>
       </c>
-      <c r="H93" t="n">
+      <c r="I93" t="n">
         <v>38430</v>
       </c>
-      <c r="I93" t="n">
+      <c r="J93" t="n">
         <v>11</v>
       </c>
     </row>
@@ -3304,22 +3579,25 @@
       <c r="C94" t="n">
         <v>1</v>
       </c>
-      <c r="D94" s="4" t="n">
+      <c r="D94" t="n">
         <v>1</v>
       </c>
-      <c r="E94" t="n">
-        <v>31</v>
+      <c r="E94" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="F94" t="n">
         <v>31</v>
       </c>
       <c r="G94" t="n">
+        <v>31</v>
+      </c>
+      <c r="H94" t="n">
         <v>62</v>
       </c>
-      <c r="H94" t="n">
+      <c r="I94" t="n">
         <v>35848</v>
       </c>
-      <c r="I94" t="n">
+      <c r="J94" t="n">
         <v>31</v>
       </c>
     </row>
@@ -3335,22 +3613,25 @@
       <c r="C95" t="n">
         <v>2</v>
       </c>
-      <c r="D95" s="4" t="n">
-        <v>0.3333333333333333</v>
-      </c>
-      <c r="E95" t="n">
-        <v>31</v>
+      <c r="D95" t="n">
+        <v>2</v>
+      </c>
+      <c r="E95" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="F95" t="n">
         <v>31</v>
       </c>
       <c r="G95" t="n">
+        <v>31</v>
+      </c>
+      <c r="H95" t="n">
         <v>62</v>
       </c>
-      <c r="H95" t="n">
+      <c r="I95" t="n">
         <v>55802</v>
       </c>
-      <c r="I95" t="n">
+      <c r="J95" t="n">
         <v>16</v>
       </c>
     </row>
@@ -3364,24 +3645,27 @@
         <v>7</v>
       </c>
       <c r="C96" t="n">
+        <v>5</v>
+      </c>
+      <c r="D96" t="n">
         <v>3</v>
       </c>
-      <c r="D96" s="4" t="n">
-        <v>0.4285714285714285</v>
-      </c>
-      <c r="E96" t="n">
+      <c r="E96" s="4" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F96" t="n">
         <v>30</v>
       </c>
-      <c r="F96" t="n">
+      <c r="G96" t="n">
         <v>29</v>
       </c>
-      <c r="G96" t="n">
+      <c r="H96" t="n">
         <v>59</v>
       </c>
-      <c r="H96" t="n">
+      <c r="I96" t="n">
         <v>44999</v>
       </c>
-      <c r="I96" t="n">
+      <c r="J96" t="n">
         <v>10</v>
       </c>
     </row>
@@ -3397,22 +3681,25 @@
       <c r="C97" t="n">
         <v>3</v>
       </c>
-      <c r="D97" s="4" t="n">
-        <v>0.3333333333333333</v>
-      </c>
-      <c r="E97" t="n">
-        <v>29</v>
+      <c r="D97" t="n">
+        <v>3</v>
+      </c>
+      <c r="E97" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="F97" t="n">
         <v>29</v>
       </c>
       <c r="G97" t="n">
+        <v>29</v>
+      </c>
+      <c r="H97" t="n">
         <v>58</v>
       </c>
-      <c r="H97" t="n">
+      <c r="I97" t="n">
         <v>45435</v>
       </c>
-      <c r="I97" t="n">
+      <c r="J97" t="n">
         <v>10</v>
       </c>
     </row>
@@ -3428,22 +3715,25 @@
       <c r="C98" t="n">
         <v>2</v>
       </c>
-      <c r="D98" s="4" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E98" t="n">
+      <c r="D98" t="n">
+        <v>2</v>
+      </c>
+      <c r="E98" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F98" t="n">
         <v>27</v>
       </c>
-      <c r="F98" t="n">
+      <c r="G98" t="n">
         <v>26</v>
       </c>
-      <c r="G98" t="n">
+      <c r="H98" t="n">
         <v>53</v>
       </c>
-      <c r="H98" t="n">
+      <c r="I98" t="n">
         <v>40774</v>
       </c>
-      <c r="I98" t="n">
+      <c r="J98" t="n">
         <v>14</v>
       </c>
     </row>
@@ -3457,24 +3747,27 @@
         <v>5</v>
       </c>
       <c r="C99" t="n">
+        <v>4</v>
+      </c>
+      <c r="D99" t="n">
         <v>3</v>
       </c>
-      <c r="D99" s="4" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="E99" t="n">
-        <v>27</v>
+      <c r="E99" s="4" t="n">
+        <v>0.75</v>
       </c>
       <c r="F99" t="n">
         <v>27</v>
       </c>
       <c r="G99" t="n">
+        <v>27</v>
+      </c>
+      <c r="H99" t="n">
         <v>54</v>
       </c>
-      <c r="H99" t="n">
+      <c r="I99" t="n">
         <v>46920</v>
       </c>
-      <c r="I99" t="n">
+      <c r="J99" t="n">
         <v>9</v>
       </c>
     </row>
@@ -3490,22 +3783,25 @@
       <c r="C100" t="n">
         <v>1</v>
       </c>
-      <c r="D100" s="4" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E100" t="n">
-        <v>27</v>
+      <c r="D100" t="n">
+        <v>1</v>
+      </c>
+      <c r="E100" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="F100" t="n">
         <v>27</v>
       </c>
       <c r="G100" t="n">
+        <v>27</v>
+      </c>
+      <c r="H100" t="n">
         <v>54</v>
       </c>
-      <c r="H100" t="n">
+      <c r="I100" t="n">
         <v>45399</v>
       </c>
-      <c r="I100" t="n">
+      <c r="J100" t="n">
         <v>27</v>
       </c>
     </row>
@@ -3519,24 +3815,27 @@
         <v>6</v>
       </c>
       <c r="C101" t="n">
+        <v>3</v>
+      </c>
+      <c r="D101" t="n">
         <v>2</v>
       </c>
-      <c r="D101" s="4" t="n">
-        <v>0.3333333333333333</v>
-      </c>
-      <c r="E101" t="n">
+      <c r="E101" s="4" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="F101" t="n">
         <v>25</v>
       </c>
-      <c r="F101" t="n">
+      <c r="G101" t="n">
         <v>24</v>
       </c>
-      <c r="G101" t="n">
+      <c r="H101" t="n">
         <v>49</v>
       </c>
-      <c r="H101" t="n">
+      <c r="I101" t="n">
         <v>27843</v>
       </c>
-      <c r="I101" t="n">
+      <c r="J101" t="n">
         <v>12</v>
       </c>
     </row>
@@ -3552,22 +3851,25 @@
       <c r="C102" t="n">
         <v>1</v>
       </c>
-      <c r="D102" s="4" t="n">
-        <v>0.1666666666666667</v>
-      </c>
-      <c r="E102" t="n">
-        <v>25</v>
+      <c r="D102" t="n">
+        <v>1</v>
+      </c>
+      <c r="E102" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="F102" t="n">
         <v>25</v>
       </c>
       <c r="G102" t="n">
+        <v>25</v>
+      </c>
+      <c r="H102" t="n">
         <v>50</v>
       </c>
-      <c r="H102" t="n">
+      <c r="I102" t="n">
         <v>37538</v>
       </c>
-      <c r="I102" t="n">
+      <c r="J102" t="n">
         <v>25</v>
       </c>
     </row>
@@ -3583,22 +3885,25 @@
       <c r="C103" t="n">
         <v>4</v>
       </c>
-      <c r="D103" s="4" t="n">
-        <v>0.1904761904761905</v>
-      </c>
-      <c r="E103" t="n">
-        <v>24</v>
+      <c r="D103" t="n">
+        <v>4</v>
+      </c>
+      <c r="E103" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="F103" t="n">
         <v>24</v>
       </c>
       <c r="G103" t="n">
+        <v>24</v>
+      </c>
+      <c r="H103" t="n">
         <v>48</v>
       </c>
-      <c r="H103" t="n">
+      <c r="I103" t="n">
         <v>35052</v>
       </c>
-      <c r="I103" t="n">
+      <c r="J103" t="n">
         <v>6</v>
       </c>
     </row>
@@ -3614,22 +3919,25 @@
       <c r="C104" t="n">
         <v>4</v>
       </c>
-      <c r="D104" s="4" t="n">
+      <c r="D104" t="n">
+        <v>4</v>
+      </c>
+      <c r="E104" s="4" t="n">
         <v>1</v>
-      </c>
-      <c r="E104" t="n">
-        <v>24</v>
       </c>
       <c r="F104" t="n">
         <v>24</v>
       </c>
       <c r="G104" t="n">
+        <v>24</v>
+      </c>
+      <c r="H104" t="n">
         <v>48</v>
       </c>
-      <c r="H104" t="n">
+      <c r="I104" t="n">
         <v>34110</v>
       </c>
-      <c r="I104" t="n">
+      <c r="J104" t="n">
         <v>6</v>
       </c>
     </row>
@@ -3643,24 +3951,27 @@
         <v>8</v>
       </c>
       <c r="C105" t="n">
+        <v>3</v>
+      </c>
+      <c r="D105" t="n">
         <v>1</v>
       </c>
-      <c r="D105" s="4" t="n">
-        <v>0.125</v>
-      </c>
-      <c r="E105" t="n">
-        <v>24</v>
+      <c r="E105" s="4" t="n">
+        <v>0.3333333333333333</v>
       </c>
       <c r="F105" t="n">
         <v>24</v>
       </c>
       <c r="G105" t="n">
+        <v>24</v>
+      </c>
+      <c r="H105" t="n">
         <v>48</v>
       </c>
-      <c r="H105" t="n">
+      <c r="I105" t="n">
         <v>27495</v>
       </c>
-      <c r="I105" t="n">
+      <c r="J105" t="n">
         <v>24</v>
       </c>
     </row>
@@ -3676,22 +3987,25 @@
       <c r="C106" t="n">
         <v>2</v>
       </c>
-      <c r="D106" s="4" t="n">
-        <v>0.3333333333333333</v>
-      </c>
-      <c r="E106" t="n">
-        <v>22</v>
+      <c r="D106" t="n">
+        <v>2</v>
+      </c>
+      <c r="E106" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="F106" t="n">
         <v>22</v>
       </c>
       <c r="G106" t="n">
+        <v>22</v>
+      </c>
+      <c r="H106" t="n">
         <v>44</v>
       </c>
-      <c r="H106" t="n">
+      <c r="I106" t="n">
         <v>26374</v>
       </c>
-      <c r="I106" t="n">
+      <c r="J106" t="n">
         <v>11</v>
       </c>
     </row>
@@ -3705,24 +4019,27 @@
         <v>3</v>
       </c>
       <c r="C107" t="n">
+        <v>3</v>
+      </c>
+      <c r="D107" t="n">
         <v>2</v>
       </c>
-      <c r="D107" s="4" t="n">
+      <c r="E107" s="4" t="n">
         <v>0.6666666666666666</v>
-      </c>
-      <c r="E107" t="n">
-        <v>21</v>
       </c>
       <c r="F107" t="n">
         <v>21</v>
       </c>
       <c r="G107" t="n">
+        <v>21</v>
+      </c>
+      <c r="H107" t="n">
         <v>42</v>
       </c>
-      <c r="H107" t="n">
+      <c r="I107" t="n">
         <v>23682</v>
       </c>
-      <c r="I107" t="n">
+      <c r="J107" t="n">
         <v>10</v>
       </c>
     </row>
@@ -3738,22 +4055,25 @@
       <c r="C108" t="n">
         <v>1</v>
       </c>
-      <c r="D108" s="4" t="n">
-        <v>0.3333333333333333</v>
-      </c>
-      <c r="E108" t="n">
-        <v>20</v>
+      <c r="D108" t="n">
+        <v>1</v>
+      </c>
+      <c r="E108" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="F108" t="n">
         <v>20</v>
       </c>
       <c r="G108" t="n">
+        <v>20</v>
+      </c>
+      <c r="H108" t="n">
         <v>40</v>
       </c>
-      <c r="H108" t="n">
+      <c r="I108" t="n">
         <v>38328</v>
       </c>
-      <c r="I108" t="n">
+      <c r="J108" t="n">
         <v>20</v>
       </c>
     </row>
@@ -3769,22 +4089,25 @@
       <c r="C109" t="n">
         <v>1</v>
       </c>
-      <c r="D109" s="4" t="n">
+      <c r="D109" t="n">
         <v>1</v>
       </c>
-      <c r="E109" t="n">
-        <v>19</v>
+      <c r="E109" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="F109" t="n">
         <v>19</v>
       </c>
       <c r="G109" t="n">
+        <v>19</v>
+      </c>
+      <c r="H109" t="n">
         <v>38</v>
       </c>
-      <c r="H109" t="n">
+      <c r="I109" t="n">
         <v>31988</v>
       </c>
-      <c r="I109" t="n">
+      <c r="J109" t="n">
         <v>19</v>
       </c>
     </row>
@@ -3798,24 +4121,27 @@
         <v>5</v>
       </c>
       <c r="C110" t="n">
+        <v>4</v>
+      </c>
+      <c r="D110" t="n">
         <v>3</v>
       </c>
-      <c r="D110" s="4" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="E110" t="n">
-        <v>19</v>
+      <c r="E110" s="4" t="n">
+        <v>0.75</v>
       </c>
       <c r="F110" t="n">
         <v>19</v>
       </c>
       <c r="G110" t="n">
+        <v>19</v>
+      </c>
+      <c r="H110" t="n">
         <v>38</v>
       </c>
-      <c r="H110" t="n">
+      <c r="I110" t="n">
         <v>32831</v>
       </c>
-      <c r="I110" t="n">
+      <c r="J110" t="n">
         <v>6</v>
       </c>
     </row>
@@ -3831,22 +4157,25 @@
       <c r="C111" t="n">
         <v>4</v>
       </c>
-      <c r="D111" s="4" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="E111" t="n">
-        <v>18</v>
+      <c r="D111" t="n">
+        <v>4</v>
+      </c>
+      <c r="E111" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="F111" t="n">
         <v>18</v>
       </c>
       <c r="G111" t="n">
+        <v>18</v>
+      </c>
+      <c r="H111" t="n">
         <v>36</v>
       </c>
-      <c r="H111" t="n">
+      <c r="I111" t="n">
         <v>32734</v>
       </c>
-      <c r="I111" t="n">
+      <c r="J111" t="n">
         <v>4</v>
       </c>
     </row>
@@ -3862,22 +4191,25 @@
       <c r="C112" t="n">
         <v>1</v>
       </c>
-      <c r="D112" s="4" t="n">
-        <v>0.3333333333333333</v>
-      </c>
-      <c r="E112" t="n">
-        <v>18</v>
+      <c r="D112" t="n">
+        <v>1</v>
+      </c>
+      <c r="E112" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="F112" t="n">
         <v>18</v>
       </c>
       <c r="G112" t="n">
+        <v>18</v>
+      </c>
+      <c r="H112" t="n">
         <v>36</v>
       </c>
-      <c r="H112" t="n">
+      <c r="I112" t="n">
         <v>25971</v>
       </c>
-      <c r="I112" t="n">
+      <c r="J112" t="n">
         <v>18</v>
       </c>
     </row>
@@ -3891,24 +4223,27 @@
         <v>6</v>
       </c>
       <c r="C113" t="n">
+        <v>2</v>
+      </c>
+      <c r="D113" t="n">
         <v>1</v>
       </c>
-      <c r="D113" s="4" t="n">
-        <v>0.1666666666666667</v>
-      </c>
-      <c r="E113" t="n">
-        <v>15</v>
+      <c r="E113" s="4" t="n">
+        <v>0.5</v>
       </c>
       <c r="F113" t="n">
         <v>15</v>
       </c>
       <c r="G113" t="n">
+        <v>15</v>
+      </c>
+      <c r="H113" t="n">
         <v>30</v>
       </c>
-      <c r="H113" t="n">
+      <c r="I113" t="n">
         <v>20108</v>
       </c>
-      <c r="I113" t="n">
+      <c r="J113" t="n">
         <v>15</v>
       </c>
     </row>
@@ -3924,22 +4259,25 @@
       <c r="C114" t="n">
         <v>1</v>
       </c>
-      <c r="D114" s="4" t="n">
+      <c r="D114" t="n">
         <v>1</v>
       </c>
-      <c r="E114" t="n">
-        <v>14</v>
+      <c r="E114" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="F114" t="n">
         <v>14</v>
       </c>
       <c r="G114" t="n">
+        <v>14</v>
+      </c>
+      <c r="H114" t="n">
         <v>28</v>
       </c>
-      <c r="H114" t="n">
+      <c r="I114" t="n">
         <v>14820</v>
       </c>
-      <c r="I114" t="n">
+      <c r="J114" t="n">
         <v>14</v>
       </c>
     </row>
@@ -3955,22 +4293,25 @@
       <c r="C115" t="n">
         <v>1</v>
       </c>
-      <c r="D115" s="4" t="n">
+      <c r="D115" t="n">
         <v>1</v>
       </c>
-      <c r="E115" t="n">
-        <v>13</v>
+      <c r="E115" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="F115" t="n">
         <v>13</v>
       </c>
       <c r="G115" t="n">
+        <v>13</v>
+      </c>
+      <c r="H115" t="n">
         <v>26</v>
       </c>
-      <c r="H115" t="n">
+      <c r="I115" t="n">
         <v>11996</v>
       </c>
-      <c r="I115" t="n">
+      <c r="J115" t="n">
         <v>13</v>
       </c>
     </row>
@@ -3986,22 +4327,25 @@
       <c r="C116" t="n">
         <v>1</v>
       </c>
-      <c r="D116" s="4" t="n">
+      <c r="D116" t="n">
         <v>1</v>
       </c>
-      <c r="E116" t="n">
-        <v>13</v>
+      <c r="E116" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="F116" t="n">
         <v>13</v>
       </c>
       <c r="G116" t="n">
+        <v>13</v>
+      </c>
+      <c r="H116" t="n">
         <v>26</v>
       </c>
-      <c r="H116" t="n">
+      <c r="I116" t="n">
         <v>19895</v>
       </c>
-      <c r="I116" t="n">
+      <c r="J116" t="n">
         <v>13</v>
       </c>
     </row>
@@ -4017,22 +4361,25 @@
       <c r="C117" t="n">
         <v>1</v>
       </c>
-      <c r="D117" s="4" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E117" t="n">
-        <v>13</v>
+      <c r="D117" t="n">
+        <v>1</v>
+      </c>
+      <c r="E117" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="F117" t="n">
         <v>13</v>
       </c>
       <c r="G117" t="n">
+        <v>13</v>
+      </c>
+      <c r="H117" t="n">
         <v>26</v>
       </c>
-      <c r="H117" t="n">
+      <c r="I117" t="n">
         <v>15588</v>
       </c>
-      <c r="I117" t="n">
+      <c r="J117" t="n">
         <v>13</v>
       </c>
     </row>
@@ -4048,22 +4395,25 @@
       <c r="C118" t="n">
         <v>4</v>
       </c>
-      <c r="D118" s="4" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="E118" t="n">
-        <v>12</v>
+      <c r="D118" t="n">
+        <v>4</v>
+      </c>
+      <c r="E118" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="F118" t="n">
         <v>12</v>
       </c>
       <c r="G118" t="n">
+        <v>12</v>
+      </c>
+      <c r="H118" t="n">
         <v>24</v>
       </c>
-      <c r="H118" t="n">
+      <c r="I118" t="n">
         <v>20290</v>
       </c>
-      <c r="I118" t="n">
+      <c r="J118" t="n">
         <v>3</v>
       </c>
     </row>
@@ -4079,22 +4429,25 @@
       <c r="C119" t="n">
         <v>1</v>
       </c>
-      <c r="D119" s="4" t="n">
+      <c r="D119" t="n">
         <v>1</v>
       </c>
-      <c r="E119" t="n">
-        <v>12</v>
+      <c r="E119" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="F119" t="n">
         <v>12</v>
       </c>
       <c r="G119" t="n">
+        <v>12</v>
+      </c>
+      <c r="H119" t="n">
         <v>24</v>
       </c>
-      <c r="H119" t="n">
+      <c r="I119" t="n">
         <v>18146</v>
       </c>
-      <c r="I119" t="n">
+      <c r="J119" t="n">
         <v>12</v>
       </c>
     </row>
@@ -4108,24 +4461,27 @@
         <v>6</v>
       </c>
       <c r="C120" t="n">
+        <v>2</v>
+      </c>
+      <c r="D120" t="n">
         <v>1</v>
       </c>
-      <c r="D120" s="4" t="n">
-        <v>0.1666666666666667</v>
-      </c>
-      <c r="E120" t="n">
+      <c r="E120" s="4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F120" t="n">
         <v>11</v>
       </c>
-      <c r="F120" t="n">
+      <c r="G120" t="n">
         <v>10</v>
       </c>
-      <c r="G120" t="n">
+      <c r="H120" t="n">
         <v>21</v>
       </c>
-      <c r="H120" t="n">
+      <c r="I120" t="n">
         <v>11363</v>
       </c>
-      <c r="I120" t="n">
+      <c r="J120" t="n">
         <v>11</v>
       </c>
     </row>
@@ -4141,22 +4497,25 @@
       <c r="C121" t="n">
         <v>1</v>
       </c>
-      <c r="D121" s="4" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E121" t="n">
+      <c r="D121" t="n">
+        <v>1</v>
+      </c>
+      <c r="E121" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F121" t="n">
         <v>10</v>
       </c>
-      <c r="F121" t="n">
+      <c r="G121" t="n">
         <v>9</v>
       </c>
-      <c r="G121" t="n">
+      <c r="H121" t="n">
         <v>19</v>
       </c>
-      <c r="H121" t="n">
+      <c r="I121" t="n">
         <v>12111</v>
       </c>
-      <c r="I121" t="n">
+      <c r="J121" t="n">
         <v>10</v>
       </c>
     </row>
@@ -4172,22 +4531,25 @@
       <c r="C122" t="n">
         <v>2</v>
       </c>
-      <c r="D122" s="4" t="n">
-        <v>0.1052631578947368</v>
-      </c>
-      <c r="E122" t="n">
-        <v>9</v>
+      <c r="D122" t="n">
+        <v>2</v>
+      </c>
+      <c r="E122" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="F122" t="n">
         <v>9</v>
       </c>
       <c r="G122" t="n">
+        <v>9</v>
+      </c>
+      <c r="H122" t="n">
         <v>18</v>
       </c>
-      <c r="H122" t="n">
+      <c r="I122" t="n">
         <v>13220</v>
       </c>
-      <c r="I122" t="n">
+      <c r="J122" t="n">
         <v>4</v>
       </c>
     </row>
@@ -4203,22 +4565,25 @@
       <c r="C123" t="n">
         <v>1</v>
       </c>
-      <c r="D123" s="4" t="n">
+      <c r="D123" t="n">
         <v>1</v>
       </c>
-      <c r="E123" t="n">
-        <v>9</v>
+      <c r="E123" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="F123" t="n">
         <v>9</v>
       </c>
       <c r="G123" t="n">
+        <v>9</v>
+      </c>
+      <c r="H123" t="n">
         <v>18</v>
       </c>
-      <c r="H123" t="n">
+      <c r="I123" t="n">
         <v>15941</v>
       </c>
-      <c r="I123" t="n">
+      <c r="J123" t="n">
         <v>9</v>
       </c>
     </row>
@@ -4234,22 +4599,25 @@
       <c r="C124" t="n">
         <v>1</v>
       </c>
-      <c r="D124" s="4" t="n">
+      <c r="D124" t="n">
         <v>1</v>
       </c>
-      <c r="E124" t="n">
-        <v>9</v>
+      <c r="E124" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="F124" t="n">
         <v>9</v>
       </c>
       <c r="G124" t="n">
+        <v>9</v>
+      </c>
+      <c r="H124" t="n">
         <v>18</v>
       </c>
-      <c r="H124" t="n">
+      <c r="I124" t="n">
         <v>13727</v>
       </c>
-      <c r="I124" t="n">
+      <c r="J124" t="n">
         <v>9</v>
       </c>
     </row>
@@ -4265,22 +4633,25 @@
       <c r="C125" t="n">
         <v>1</v>
       </c>
-      <c r="D125" s="4" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E125" t="n">
-        <v>8</v>
+      <c r="D125" t="n">
+        <v>1</v>
+      </c>
+      <c r="E125" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="F125" t="n">
         <v>8</v>
       </c>
       <c r="G125" t="n">
+        <v>8</v>
+      </c>
+      <c r="H125" t="n">
         <v>16</v>
       </c>
-      <c r="H125" t="n">
+      <c r="I125" t="n">
         <v>18271</v>
       </c>
-      <c r="I125" t="n">
+      <c r="J125" t="n">
         <v>8</v>
       </c>
     </row>
@@ -4294,24 +4665,27 @@
         <v>6</v>
       </c>
       <c r="C126" t="n">
+        <v>6</v>
+      </c>
+      <c r="D126" t="n">
         <v>3</v>
       </c>
-      <c r="D126" s="4" t="n">
+      <c r="E126" s="4" t="n">
         <v>0.5</v>
-      </c>
-      <c r="E126" t="n">
-        <v>7</v>
       </c>
       <c r="F126" t="n">
         <v>7</v>
       </c>
       <c r="G126" t="n">
+        <v>7</v>
+      </c>
+      <c r="H126" t="n">
         <v>14</v>
       </c>
-      <c r="H126" t="n">
+      <c r="I126" t="n">
         <v>6662</v>
       </c>
-      <c r="I126" t="n">
+      <c r="J126" t="n">
         <v>2</v>
       </c>
     </row>
@@ -4327,22 +4701,25 @@
       <c r="C127" t="n">
         <v>1</v>
       </c>
-      <c r="D127" s="4" t="n">
-        <v>0.3333333333333333</v>
-      </c>
-      <c r="E127" t="n">
-        <v>7</v>
+      <c r="D127" t="n">
+        <v>1</v>
+      </c>
+      <c r="E127" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="F127" t="n">
         <v>7</v>
       </c>
       <c r="G127" t="n">
+        <v>7</v>
+      </c>
+      <c r="H127" t="n">
         <v>14</v>
       </c>
-      <c r="H127" t="n">
+      <c r="I127" t="n">
         <v>9215</v>
       </c>
-      <c r="I127" t="n">
+      <c r="J127" t="n">
         <v>7</v>
       </c>
     </row>
@@ -4358,22 +4735,25 @@
       <c r="C128" t="n">
         <v>1</v>
       </c>
-      <c r="D128" s="4" t="n">
+      <c r="D128" t="n">
         <v>1</v>
       </c>
-      <c r="E128" t="n">
-        <v>6</v>
+      <c r="E128" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="F128" t="n">
         <v>6</v>
       </c>
       <c r="G128" t="n">
+        <v>6</v>
+      </c>
+      <c r="H128" t="n">
         <v>12</v>
       </c>
-      <c r="H128" t="n">
+      <c r="I128" t="n">
         <v>7289</v>
       </c>
-      <c r="I128" t="n">
+      <c r="J128" t="n">
         <v>6</v>
       </c>
     </row>
@@ -4387,24 +4767,27 @@
         <v>9</v>
       </c>
       <c r="C129" t="n">
+        <v>4</v>
+      </c>
+      <c r="D129" t="n">
         <v>2</v>
       </c>
-      <c r="D129" s="4" t="n">
-        <v>0.2222222222222222</v>
-      </c>
-      <c r="E129" t="n">
-        <v>6</v>
+      <c r="E129" s="4" t="n">
+        <v>0.5</v>
       </c>
       <c r="F129" t="n">
         <v>6</v>
       </c>
       <c r="G129" t="n">
+        <v>6</v>
+      </c>
+      <c r="H129" t="n">
         <v>12</v>
       </c>
-      <c r="H129" t="n">
+      <c r="I129" t="n">
         <v>9240</v>
       </c>
-      <c r="I129" t="n">
+      <c r="J129" t="n">
         <v>3</v>
       </c>
     </row>
@@ -4418,24 +4801,27 @@
         <v>4</v>
       </c>
       <c r="C130" t="n">
+        <v>3</v>
+      </c>
+      <c r="D130" t="n">
         <v>2</v>
       </c>
-      <c r="D130" s="4" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E130" t="n">
-        <v>6</v>
+      <c r="E130" s="4" t="n">
+        <v>0.6666666666666666</v>
       </c>
       <c r="F130" t="n">
         <v>6</v>
       </c>
       <c r="G130" t="n">
+        <v>6</v>
+      </c>
+      <c r="H130" t="n">
         <v>12</v>
       </c>
-      <c r="H130" t="n">
+      <c r="I130" t="n">
         <v>9099</v>
       </c>
-      <c r="I130" t="n">
+      <c r="J130" t="n">
         <v>3</v>
       </c>
     </row>
@@ -4451,22 +4837,25 @@
       <c r="C131" t="n">
         <v>2</v>
       </c>
-      <c r="D131" s="4" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="E131" t="n">
-        <v>5</v>
+      <c r="D131" t="n">
+        <v>2</v>
+      </c>
+      <c r="E131" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="F131" t="n">
         <v>5</v>
       </c>
       <c r="G131" t="n">
+        <v>5</v>
+      </c>
+      <c r="H131" t="n">
         <v>10</v>
       </c>
-      <c r="H131" t="n">
+      <c r="I131" t="n">
         <v>7956</v>
       </c>
-      <c r="I131" t="n">
+      <c r="J131" t="n">
         <v>2</v>
       </c>
     </row>
@@ -4482,22 +4871,25 @@
       <c r="C132" t="n">
         <v>1</v>
       </c>
-      <c r="D132" s="4" t="n">
-        <v>0.1111111111111111</v>
-      </c>
-      <c r="E132" t="n">
-        <v>5</v>
+      <c r="D132" t="n">
+        <v>1</v>
+      </c>
+      <c r="E132" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="F132" t="n">
         <v>5</v>
       </c>
       <c r="G132" t="n">
+        <v>5</v>
+      </c>
+      <c r="H132" t="n">
         <v>10</v>
       </c>
-      <c r="H132" t="n">
+      <c r="I132" t="n">
         <v>6256</v>
       </c>
-      <c r="I132" t="n">
+      <c r="J132" t="n">
         <v>5</v>
       </c>
     </row>
@@ -4513,22 +4905,25 @@
       <c r="C133" t="n">
         <v>1</v>
       </c>
-      <c r="D133" s="4" t="n">
-        <v>0.1428571428571428</v>
-      </c>
-      <c r="E133" t="n">
-        <v>5</v>
+      <c r="D133" t="n">
+        <v>1</v>
+      </c>
+      <c r="E133" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="F133" t="n">
         <v>5</v>
       </c>
       <c r="G133" t="n">
+        <v>5</v>
+      </c>
+      <c r="H133" t="n">
         <v>10</v>
       </c>
-      <c r="H133" t="n">
+      <c r="I133" t="n">
         <v>8632</v>
       </c>
-      <c r="I133" t="n">
+      <c r="J133" t="n">
         <v>5</v>
       </c>
     </row>
@@ -4542,24 +4937,27 @@
         <v>8</v>
       </c>
       <c r="C134" t="n">
+        <v>2</v>
+      </c>
+      <c r="D134" t="n">
         <v>1</v>
       </c>
-      <c r="D134" s="4" t="n">
-        <v>0.125</v>
-      </c>
-      <c r="E134" t="n">
-        <v>4</v>
+      <c r="E134" s="4" t="n">
+        <v>0.5</v>
       </c>
       <c r="F134" t="n">
         <v>4</v>
       </c>
       <c r="G134" t="n">
+        <v>4</v>
+      </c>
+      <c r="H134" t="n">
         <v>8</v>
       </c>
-      <c r="H134" t="n">
+      <c r="I134" t="n">
         <v>6316</v>
       </c>
-      <c r="I134" t="n">
+      <c r="J134" t="n">
         <v>4</v>
       </c>
     </row>
@@ -4575,22 +4973,25 @@
       <c r="C135" t="n">
         <v>1</v>
       </c>
-      <c r="D135" s="4" t="n">
+      <c r="D135" t="n">
         <v>1</v>
       </c>
-      <c r="E135" t="n">
-        <v>3</v>
+      <c r="E135" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="F135" t="n">
         <v>3</v>
       </c>
       <c r="G135" t="n">
+        <v>3</v>
+      </c>
+      <c r="H135" t="n">
         <v>6</v>
       </c>
-      <c r="H135" t="n">
+      <c r="I135" t="n">
         <v>3415</v>
       </c>
-      <c r="I135" t="n">
+      <c r="J135" t="n">
         <v>3</v>
       </c>
     </row>
@@ -4606,22 +5007,25 @@
       <c r="C136" t="n">
         <v>2</v>
       </c>
-      <c r="D136" s="4" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="E136" t="n">
-        <v>3</v>
+      <c r="D136" t="n">
+        <v>2</v>
+      </c>
+      <c r="E136" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="F136" t="n">
         <v>3</v>
       </c>
       <c r="G136" t="n">
+        <v>3</v>
+      </c>
+      <c r="H136" t="n">
         <v>6</v>
       </c>
-      <c r="H136" t="n">
+      <c r="I136" t="n">
         <v>5725</v>
       </c>
-      <c r="I136" t="n">
+      <c r="J136" t="n">
         <v>2</v>
       </c>
     </row>
@@ -4637,22 +5041,25 @@
       <c r="C137" t="n">
         <v>1</v>
       </c>
-      <c r="D137" s="4" t="n">
+      <c r="D137" t="n">
         <v>1</v>
       </c>
-      <c r="E137" t="n">
-        <v>3</v>
+      <c r="E137" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="F137" t="n">
         <v>3</v>
       </c>
       <c r="G137" t="n">
+        <v>3</v>
+      </c>
+      <c r="H137" t="n">
         <v>6</v>
       </c>
-      <c r="H137" t="n">
+      <c r="I137" t="n">
         <v>6067</v>
       </c>
-      <c r="I137" t="n">
+      <c r="J137" t="n">
         <v>3</v>
       </c>
     </row>
@@ -4668,22 +5075,25 @@
       <c r="C138" t="n">
         <v>1</v>
       </c>
-      <c r="D138" s="4" t="n">
+      <c r="D138" t="n">
         <v>1</v>
       </c>
-      <c r="E138" t="n">
-        <v>2</v>
+      <c r="E138" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="F138" t="n">
         <v>2</v>
       </c>
       <c r="G138" t="n">
+        <v>2</v>
+      </c>
+      <c r="H138" t="n">
         <v>4</v>
       </c>
-      <c r="H138" t="n">
+      <c r="I138" t="n">
         <v>3262</v>
       </c>
-      <c r="I138" t="n">
+      <c r="J138" t="n">
         <v>2</v>
       </c>
     </row>
@@ -4699,22 +5109,25 @@
       <c r="C139" t="n">
         <v>1</v>
       </c>
-      <c r="D139" s="4" t="n">
+      <c r="D139" t="n">
         <v>1</v>
       </c>
-      <c r="E139" t="n">
-        <v>2</v>
+      <c r="E139" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="F139" t="n">
         <v>2</v>
       </c>
       <c r="G139" t="n">
+        <v>2</v>
+      </c>
+      <c r="H139" t="n">
         <v>4</v>
       </c>
-      <c r="H139" t="n">
+      <c r="I139" t="n">
         <v>3400</v>
       </c>
-      <c r="I139" t="n">
+      <c r="J139" t="n">
         <v>2</v>
       </c>
     </row>
@@ -4730,22 +5143,25 @@
       <c r="C140" t="n">
         <v>1</v>
       </c>
-      <c r="D140" s="4" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="E140" t="n">
+      <c r="D140" t="n">
+        <v>1</v>
+      </c>
+      <c r="E140" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F140" t="n">
         <v>1</v>
       </c>
       <c r="G140" t="n">
+        <v>1</v>
+      </c>
+      <c r="H140" t="n">
         <v>2</v>
       </c>
-      <c r="H140" t="n">
+      <c r="I140" t="n">
         <v>909</v>
       </c>
-      <c r="I140" t="n">
+      <c r="J140" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Revert 部署別集計 usage_rate divisor back to 登録者数(全体)
ユーザー指示により、利用率=利用者数÷登録者数(全体)に変更。
登録者数(利用開始済み)の列は引き続き参考情報として併記する。

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01598FP6oS2STFUTDPWRj1o6
</commit_message>
<xml_diff>
--- a/QommonsAI利用集計.xlsx
+++ b/QommonsAI利用集計.xlsx
@@ -482,7 +482,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>集計期間: 2026-07-01 〜 2026-07-22  ／ 利用回数=プロンプト(質問)数  ／ 使用文字数=入力+出力(プレフィックス除く)  ／ 利用率=利用者数÷登録者数(利用開始済み)</t>
+          <t>集計期間: 2026-07-01 〜 2026-07-22  ／ 利用回数=プロンプト(質問)数  ／ 使用文字数=入力+出力(プレフィックス除く)  ／ 利用率=利用者数÷登録者数(全体)</t>
         </is>
       </c>
     </row>
@@ -591,7 +591,7 @@
         <v>11</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>1</v>
+        <v>0.8461538461538461</v>
       </c>
       <c r="F6" t="n">
         <v>1132</v>
@@ -659,7 +659,7 @@
         <v>10</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>1</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="F8" t="n">
         <v>816</v>
@@ -693,7 +693,7 @@
         <v>13</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>0.8125</v>
+        <v>0.7647058823529411</v>
       </c>
       <c r="F9" t="n">
         <v>688</v>
@@ -727,7 +727,7 @@
         <v>17</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>0.8095238095238095</v>
+        <v>0.5666666666666667</v>
       </c>
       <c r="F10" t="n">
         <v>674</v>
@@ -795,7 +795,7 @@
         <v>5</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>1</v>
+        <v>0.5555555555555556</v>
       </c>
       <c r="F12" t="n">
         <v>527</v>
@@ -829,7 +829,7 @@
         <v>13</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>0.8666666666666667</v>
+        <v>0.8125</v>
       </c>
       <c r="F13" t="n">
         <v>504</v>
@@ -863,7 +863,7 @@
         <v>6</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>1</v>
+        <v>0.8571428571428571</v>
       </c>
       <c r="F14" t="n">
         <v>500</v>
@@ -897,7 +897,7 @@
         <v>3</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>1</v>
+        <v>0.4285714285714285</v>
       </c>
       <c r="F15" t="n">
         <v>495</v>
@@ -931,7 +931,7 @@
         <v>8</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>0.8888888888888888</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="F16" t="n">
         <v>391</v>
@@ -965,7 +965,7 @@
         <v>8</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>1</v>
+        <v>0.8888888888888888</v>
       </c>
       <c r="F17" t="n">
         <v>368</v>
@@ -1033,7 +1033,7 @@
         <v>1</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F19" t="n">
         <v>348</v>
@@ -1067,7 +1067,7 @@
         <v>8</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>0.8</v>
+        <v>0.7272727272727273</v>
       </c>
       <c r="F20" t="n">
         <v>334</v>
@@ -1101,7 +1101,7 @@
         <v>9</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>0.8181818181818182</v>
+        <v>0.6923076923076923</v>
       </c>
       <c r="F21" t="n">
         <v>318</v>
@@ -1135,7 +1135,7 @@
         <v>9</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>0.5625</v>
+        <v>0.36</v>
       </c>
       <c r="F22" t="n">
         <v>308</v>
@@ -1169,7 +1169,7 @@
         <v>4</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>0.8</v>
+        <v>0.5714285714285714</v>
       </c>
       <c r="F23" t="n">
         <v>293</v>
@@ -1203,7 +1203,7 @@
         <v>6</v>
       </c>
       <c r="E24" s="4" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="F24" t="n">
         <v>258</v>
@@ -1237,7 +1237,7 @@
         <v>12</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>0.75</v>
+        <v>0.5714285714285714</v>
       </c>
       <c r="F25" t="n">
         <v>247</v>
@@ -1271,7 +1271,7 @@
         <v>4</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="F26" t="n">
         <v>245</v>
@@ -1305,7 +1305,7 @@
         <v>5</v>
       </c>
       <c r="E27" s="4" t="n">
-        <v>0.625</v>
+        <v>0.5</v>
       </c>
       <c r="F27" t="n">
         <v>222</v>
@@ -1339,7 +1339,7 @@
         <v>9</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>0.8181818181818182</v>
+        <v>0.5</v>
       </c>
       <c r="F28" t="n">
         <v>219</v>
@@ -1407,7 +1407,7 @@
         <v>5</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.7142857142857143</v>
       </c>
       <c r="F30" t="n">
         <v>171</v>
@@ -1441,7 +1441,7 @@
         <v>2</v>
       </c>
       <c r="E31" s="4" t="n">
-        <v>1</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="F31" t="n">
         <v>163</v>
@@ -1475,7 +1475,7 @@
         <v>5</v>
       </c>
       <c r="E32" s="4" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F32" t="n">
         <v>155</v>
@@ -1509,7 +1509,7 @@
         <v>3</v>
       </c>
       <c r="E33" s="4" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F33" t="n">
         <v>154</v>
@@ -1577,7 +1577,7 @@
         <v>8</v>
       </c>
       <c r="E35" s="4" t="n">
-        <v>1</v>
+        <v>0.8888888888888888</v>
       </c>
       <c r="F35" t="n">
         <v>143</v>
@@ -1611,7 +1611,7 @@
         <v>2</v>
       </c>
       <c r="E36" s="4" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.5</v>
       </c>
       <c r="F36" t="n">
         <v>136</v>
@@ -1645,7 +1645,7 @@
         <v>3</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="F37" t="n">
         <v>130</v>
@@ -1713,7 +1713,7 @@
         <v>6</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>1</v>
+        <v>0.8571428571428571</v>
       </c>
       <c r="F39" t="n">
         <v>125</v>
@@ -1747,7 +1747,7 @@
         <v>4</v>
       </c>
       <c r="E40" s="4" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.5</v>
       </c>
       <c r="F40" t="n">
         <v>124</v>
@@ -1781,7 +1781,7 @@
         <v>4</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>0.8</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="F41" t="n">
         <v>120</v>
@@ -1815,7 +1815,7 @@
         <v>5</v>
       </c>
       <c r="E42" s="4" t="n">
-        <v>1</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="F42" t="n">
         <v>118</v>
@@ -1849,7 +1849,7 @@
         <v>6</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>1</v>
+        <v>0.8571428571428571</v>
       </c>
       <c r="F43" t="n">
         <v>116</v>
@@ -1883,7 +1883,7 @@
         <v>5</v>
       </c>
       <c r="E44" s="4" t="n">
-        <v>1</v>
+        <v>0.625</v>
       </c>
       <c r="F44" t="n">
         <v>115</v>
@@ -1917,7 +1917,7 @@
         <v>4</v>
       </c>
       <c r="E45" s="4" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.4444444444444444</v>
       </c>
       <c r="F45" t="n">
         <v>108</v>
@@ -1951,7 +1951,7 @@
         <v>6</v>
       </c>
       <c r="E46" s="4" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="F46" t="n">
         <v>106</v>
@@ -2019,7 +2019,7 @@
         <v>3</v>
       </c>
       <c r="E48" s="4" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="F48" t="n">
         <v>102</v>
@@ -2053,7 +2053,7 @@
         <v>6</v>
       </c>
       <c r="E49" s="4" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="F49" t="n">
         <v>101</v>
@@ -2087,7 +2087,7 @@
         <v>3</v>
       </c>
       <c r="E50" s="4" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F50" t="n">
         <v>101</v>
@@ -2121,7 +2121,7 @@
         <v>5</v>
       </c>
       <c r="E51" s="4" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.625</v>
       </c>
       <c r="F51" t="n">
         <v>100</v>
@@ -2155,7 +2155,7 @@
         <v>4</v>
       </c>
       <c r="E52" s="4" t="n">
-        <v>1</v>
+        <v>0.5714285714285714</v>
       </c>
       <c r="F52" t="n">
         <v>98</v>
@@ -2223,7 +2223,7 @@
         <v>7</v>
       </c>
       <c r="E54" s="4" t="n">
-        <v>0.875</v>
+        <v>0.6363636363636364</v>
       </c>
       <c r="F54" t="n">
         <v>94</v>
@@ -2257,7 +2257,7 @@
         <v>6</v>
       </c>
       <c r="E55" s="4" t="n">
-        <v>0.8571428571428571</v>
+        <v>0.5</v>
       </c>
       <c r="F55" t="n">
         <v>93</v>
@@ -2325,7 +2325,7 @@
         <v>6</v>
       </c>
       <c r="E57" s="4" t="n">
-        <v>1</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="F57" t="n">
         <v>89</v>
@@ -2359,7 +2359,7 @@
         <v>4</v>
       </c>
       <c r="E58" s="4" t="n">
-        <v>1</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="F58" t="n">
         <v>81</v>
@@ -2393,7 +2393,7 @@
         <v>5</v>
       </c>
       <c r="E59" s="4" t="n">
-        <v>1</v>
+        <v>0.625</v>
       </c>
       <c r="F59" t="n">
         <v>77</v>
@@ -2427,7 +2427,7 @@
         <v>4</v>
       </c>
       <c r="E60" s="4" t="n">
-        <v>0.5</v>
+        <v>0.4444444444444444</v>
       </c>
       <c r="F60" t="n">
         <v>74</v>
@@ -2461,7 +2461,7 @@
         <v>2</v>
       </c>
       <c r="E61" s="4" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F61" t="n">
         <v>73</v>
@@ -2495,7 +2495,7 @@
         <v>3</v>
       </c>
       <c r="E62" s="4" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F62" t="n">
         <v>71</v>
@@ -2529,7 +2529,7 @@
         <v>2</v>
       </c>
       <c r="E63" s="4" t="n">
-        <v>0.5</v>
+        <v>0.25</v>
       </c>
       <c r="F63" t="n">
         <v>70</v>
@@ -2597,7 +2597,7 @@
         <v>5</v>
       </c>
       <c r="E65" s="4" t="n">
-        <v>0.7142857142857143</v>
+        <v>0.3571428571428572</v>
       </c>
       <c r="F65" t="n">
         <v>66</v>
@@ -2631,7 +2631,7 @@
         <v>1</v>
       </c>
       <c r="E66" s="4" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F66" t="n">
         <v>66</v>
@@ -2665,7 +2665,7 @@
         <v>2</v>
       </c>
       <c r="E67" s="4" t="n">
-        <v>1</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="F67" t="n">
         <v>66</v>
@@ -2699,7 +2699,7 @@
         <v>4</v>
       </c>
       <c r="E68" s="4" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.4</v>
       </c>
       <c r="F68" t="n">
         <v>65</v>
@@ -2767,7 +2767,7 @@
         <v>3</v>
       </c>
       <c r="E70" s="4" t="n">
-        <v>0.75</v>
+        <v>0.4285714285714285</v>
       </c>
       <c r="F70" t="n">
         <v>64</v>
@@ -2801,7 +2801,7 @@
         <v>5</v>
       </c>
       <c r="E71" s="4" t="n">
-        <v>1</v>
+        <v>0.2631578947368421</v>
       </c>
       <c r="F71" t="n">
         <v>64</v>
@@ -2937,7 +2937,7 @@
         <v>2</v>
       </c>
       <c r="E75" s="4" t="n">
-        <v>1</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="F75" t="n">
         <v>59</v>
@@ -2971,7 +2971,7 @@
         <v>1</v>
       </c>
       <c r="E76" s="4" t="n">
-        <v>1</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="F76" t="n">
         <v>59</v>
@@ -3005,7 +3005,7 @@
         <v>3</v>
       </c>
       <c r="E77" s="4" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="F77" t="n">
         <v>57</v>
@@ -3039,7 +3039,7 @@
         <v>8</v>
       </c>
       <c r="E78" s="4" t="n">
-        <v>0.8</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="F78" t="n">
         <v>56</v>
@@ -3073,7 +3073,7 @@
         <v>1</v>
       </c>
       <c r="E79" s="4" t="n">
-        <v>0.5</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="F79" t="n">
         <v>56</v>
@@ -3141,7 +3141,7 @@
         <v>3</v>
       </c>
       <c r="E81" s="4" t="n">
-        <v>0.5</v>
+        <v>0.375</v>
       </c>
       <c r="F81" t="n">
         <v>55</v>
@@ -3175,7 +3175,7 @@
         <v>1</v>
       </c>
       <c r="E82" s="4" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F82" t="n">
         <v>55</v>
@@ -3209,7 +3209,7 @@
         <v>5</v>
       </c>
       <c r="E83" s="4" t="n">
-        <v>0.7142857142857143</v>
+        <v>0.4545454545454545</v>
       </c>
       <c r="F83" t="n">
         <v>51</v>
@@ -3243,7 +3243,7 @@
         <v>1</v>
       </c>
       <c r="E84" s="4" t="n">
-        <v>1</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="F84" t="n">
         <v>45</v>
@@ -3311,7 +3311,7 @@
         <v>1</v>
       </c>
       <c r="E86" s="4" t="n">
-        <v>0.5</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="F86" t="n">
         <v>42</v>
@@ -3379,7 +3379,7 @@
         <v>2</v>
       </c>
       <c r="E88" s="4" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F88" t="n">
         <v>38</v>
@@ -3413,7 +3413,7 @@
         <v>4</v>
       </c>
       <c r="E89" s="4" t="n">
-        <v>1</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="F89" t="n">
         <v>38</v>
@@ -3447,7 +3447,7 @@
         <v>1</v>
       </c>
       <c r="E90" s="4" t="n">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="F90" t="n">
         <v>37</v>
@@ -3481,7 +3481,7 @@
         <v>2</v>
       </c>
       <c r="E91" s="4" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F91" t="n">
         <v>36</v>
@@ -3515,7 +3515,7 @@
         <v>3</v>
       </c>
       <c r="E92" s="4" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="F92" t="n">
         <v>36</v>
@@ -3549,7 +3549,7 @@
         <v>3</v>
       </c>
       <c r="E93" s="4" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="F93" t="n">
         <v>36</v>
@@ -3583,7 +3583,7 @@
         <v>3</v>
       </c>
       <c r="E94" s="4" t="n">
-        <v>0.6</v>
+        <v>0.4285714285714285</v>
       </c>
       <c r="F94" t="n">
         <v>32</v>
@@ -3617,7 +3617,7 @@
         <v>1</v>
       </c>
       <c r="E95" s="4" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F95" t="n">
         <v>32</v>
@@ -3685,7 +3685,7 @@
         <v>3</v>
       </c>
       <c r="E97" s="4" t="n">
-        <v>1</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="F97" t="n">
         <v>31</v>
@@ -3719,7 +3719,7 @@
         <v>2</v>
       </c>
       <c r="E98" s="4" t="n">
-        <v>1</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="F98" t="n">
         <v>31</v>
@@ -3753,7 +3753,7 @@
         <v>2</v>
       </c>
       <c r="E99" s="4" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F99" t="n">
         <v>28</v>
@@ -3787,7 +3787,7 @@
         <v>3</v>
       </c>
       <c r="E100" s="4" t="n">
-        <v>0.75</v>
+        <v>0.6</v>
       </c>
       <c r="F100" t="n">
         <v>28</v>
@@ -3855,7 +3855,7 @@
         <v>2</v>
       </c>
       <c r="E102" s="4" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="F102" t="n">
         <v>26</v>
@@ -3889,7 +3889,7 @@
         <v>1</v>
       </c>
       <c r="E103" s="4" t="n">
-        <v>1</v>
+        <v>0.1666666666666667</v>
       </c>
       <c r="F103" t="n">
         <v>26</v>
@@ -3923,7 +3923,7 @@
         <v>1</v>
       </c>
       <c r="E104" s="4" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.125</v>
       </c>
       <c r="F104" t="n">
         <v>25</v>
@@ -3957,7 +3957,7 @@
         <v>2</v>
       </c>
       <c r="E105" s="4" t="n">
-        <v>1</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="F105" t="n">
         <v>25</v>
@@ -3991,7 +3991,7 @@
         <v>4</v>
       </c>
       <c r="E106" s="4" t="n">
-        <v>1</v>
+        <v>0.1904761904761905</v>
       </c>
       <c r="F106" t="n">
         <v>24</v>
@@ -4093,7 +4093,7 @@
         <v>1</v>
       </c>
       <c r="E109" s="4" t="n">
-        <v>1</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="F109" t="n">
         <v>20</v>
@@ -4127,7 +4127,7 @@
         <v>3</v>
       </c>
       <c r="E110" s="4" t="n">
-        <v>0.75</v>
+        <v>0.6</v>
       </c>
       <c r="F110" t="n">
         <v>19</v>
@@ -4161,7 +4161,7 @@
         <v>4</v>
       </c>
       <c r="E111" s="4" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="F111" t="n">
         <v>18</v>
@@ -4195,7 +4195,7 @@
         <v>1</v>
       </c>
       <c r="E112" s="4" t="n">
-        <v>1</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="F112" t="n">
         <v>18</v>
@@ -4229,7 +4229,7 @@
         <v>2</v>
       </c>
       <c r="E113" s="4" t="n">
-        <v>1</v>
+        <v>0.25</v>
       </c>
       <c r="F113" t="n">
         <v>15</v>
@@ -4263,7 +4263,7 @@
         <v>1</v>
       </c>
       <c r="E114" s="4" t="n">
-        <v>0.5</v>
+        <v>0.1666666666666667</v>
       </c>
       <c r="F114" t="n">
         <v>15</v>
@@ -4331,7 +4331,7 @@
         <v>4</v>
       </c>
       <c r="E116" s="4" t="n">
-        <v>1</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="F116" t="n">
         <v>13</v>
@@ -4433,7 +4433,7 @@
         <v>1</v>
       </c>
       <c r="E119" s="4" t="n">
-        <v>0.5</v>
+        <v>0.1666666666666667</v>
       </c>
       <c r="F119" t="n">
         <v>13</v>
@@ -4467,7 +4467,7 @@
         <v>1</v>
       </c>
       <c r="E120" s="4" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F120" t="n">
         <v>13</v>
@@ -4501,7 +4501,7 @@
         <v>1</v>
       </c>
       <c r="E121" s="4" t="n">
-        <v>1</v>
+        <v>0.1111111111111111</v>
       </c>
       <c r="F121" t="n">
         <v>13</v>
@@ -4569,7 +4569,7 @@
         <v>2</v>
       </c>
       <c r="E123" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F123" t="n">
         <v>12</v>
@@ -4637,7 +4637,7 @@
         <v>2</v>
       </c>
       <c r="E125" s="4" t="n">
-        <v>0.5</v>
+        <v>0.2222222222222222</v>
       </c>
       <c r="F125" t="n">
         <v>10</v>
@@ -4671,7 +4671,7 @@
         <v>2</v>
       </c>
       <c r="E126" s="4" t="n">
-        <v>1</v>
+        <v>0.1052631578947368</v>
       </c>
       <c r="F126" t="n">
         <v>9</v>
@@ -4773,7 +4773,7 @@
         <v>1</v>
       </c>
       <c r="E129" s="4" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F129" t="n">
         <v>8</v>
@@ -4807,7 +4807,7 @@
         <v>2</v>
       </c>
       <c r="E130" s="4" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="F130" t="n">
         <v>8</v>
@@ -4841,7 +4841,7 @@
         <v>1</v>
       </c>
       <c r="E131" s="4" t="n">
-        <v>1</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="F131" t="n">
         <v>7</v>
@@ -4909,7 +4909,7 @@
         <v>2</v>
       </c>
       <c r="E133" s="4" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.5</v>
       </c>
       <c r="F133" t="n">
         <v>6</v>
@@ -4943,7 +4943,7 @@
         <v>1</v>
       </c>
       <c r="E134" s="4" t="n">
-        <v>0.5</v>
+        <v>0.125</v>
       </c>
       <c r="F134" t="n">
         <v>6</v>
@@ -4977,7 +4977,7 @@
         <v>1</v>
       </c>
       <c r="E135" s="4" t="n">
-        <v>1</v>
+        <v>0.1428571428571428</v>
       </c>
       <c r="F135" t="n">
         <v>5</v>
@@ -5079,7 +5079,7 @@
         <v>2</v>
       </c>
       <c r="E138" s="4" t="n">
-        <v>1</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="F138" t="n">
         <v>3</v>
@@ -5113,7 +5113,7 @@
         <v>1</v>
       </c>
       <c r="E139" s="4" t="n">
-        <v>1</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="F139" t="n">
         <v>3</v>
@@ -5215,7 +5215,7 @@
         <v>1</v>
       </c>
       <c r="E142" s="4" t="n">
-        <v>1</v>
+        <v>0.25</v>
       </c>
       <c r="F142" t="n">
         <v>1</v>

</xml_diff>